<commit_message>
Relabel 1904-description field; Jim cleans up monument notes content
"From 1904 description" -> "In 1904 description" so cells that just
say "no" (not in the 1904 book) read as a sensible answer. Jim also
worked through a content-review checklist directly in the sheet:
corrected 2 monuments from Documented to Not Found (notes described
an actual search, not just no visit), fixed several typos, and
clarified a couple of ambiguous notes.
</commit_message>
<xml_diff>
--- a/Acton Bounds.xlsx
+++ b/Acton Bounds.xlsx
@@ -456,7 +456,7 @@
     <t>roadstone on the northeasterly side of Bear Hill road</t>
   </si>
   <si>
-    <t>looked where a private road crosses the boundary (but no bounds were found there). These coodinates are where that road crosses the border.</t>
+    <t>looked where a private road crosses the boundary (but no bounds were found there). These coordinates are where that road crosses the border.</t>
   </si>
   <si>
     <t xml:space="preserve">map estimate </t>
@@ -468,7 +468,7 @@
     <t>-71.409332</t>
   </si>
   <si>
-    <t>Bay  Drive (East)</t>
+    <t>Bay Drive (East)</t>
   </si>
   <si>
     <t>Are these public ways? May not be required</t>
@@ -529,16 +529,16 @@
     <t>Bobby's Ranch</t>
   </si>
   <si>
-    <t>Visible from the southeast corner of the fenced in area behind the main barm of Bobby's Ranch</t>
+    <t>Visible from the southeast corner of the fenced in area behind the main barn of Bobby's Ranch</t>
   </si>
   <si>
     <t>a rough split granite monument, triangular In shape, marked A L W 1832, and situated in low woodland near an open meadow, about 800 feet northwest of a cart path leading northeasterly from Nagog pond and about 2,500 feet distant from the pond;</t>
   </si>
   <si>
-    <t>Contact owners at Bobby's Ranch before any visit. You need towalk through barn, and electricity to fence needs to be turned off.</t>
-  </si>
-  <si>
-    <t>same as Nashoba Road corner?</t>
+    <t>Contact owners at Bobby's Ranch before any visit. You need to walk through barn, and electricity to fence needs to be turned off.</t>
+  </si>
+  <si>
+    <t>Maybe never installed because it would have been so close to the Acton/Littleton monument?</t>
   </si>
   <si>
     <t>42.52252</t>
@@ -559,7 +559,7 @@
     <t>next to stone wall near end of Nashoba Road</t>
   </si>
   <si>
-    <t>corner 1, a rough split granite monument of irregular shape marked A L 1831 and situated at the northerly end of Nagog pond, on the northeasterly side of the road leading from North Acton to Littletown;</t>
+    <t>corner 1, a rough split granite monument of irregular shape marked A L 1831 and situated at the northerly end of Nagog pond, on the northeasterly side of the road leading from North Acton to Littletown[sic]</t>
   </si>
   <si>
     <t>lying on ground. Too difficult to paint. Will seek to get it rescued.</t>
@@ -577,7 +577,7 @@
     <t>Nagog Pond South Shore</t>
   </si>
   <si>
-    <t>near bottom of AWD land. roughly follow tree acros path near pond uphill</t>
+    <t>near bottom of AWD land. roughly follow tree across path near pond uphill</t>
   </si>
   <si>
     <t>corner 2, a rough split granite monument of irregular shape marked A L 1831, and situated in heavy maple, oak and chestnut woods, about 288 feet from the southwesterly shore of Nagog pond.</t>
@@ -679,13 +679,13 @@
     <t>Central Street</t>
   </si>
   <si>
-    <t>Rte 2 Exit 115 (Newtown/Central</t>
-  </si>
-  <si>
-    <t>looked a couple of times, not found yet. Boxborough reports it is missing</t>
-  </si>
-  <si>
-    <t>..a rough split granite monument, triangular in shape, marked A B L. and situated at a junction of walls, about one-half mile southwest of Fort pond and about 680 feet southeast of the West Acton road;</t>
+    <t>Rte 2 Exit 115 (Newtown/Central Street)</t>
+  </si>
+  <si>
+    <t>looked a couple of times, not found yet. Boxborough reports it is missing. I think it would be in the grassy area between lanes of the exits. Unlikely to survive the construction of Rte 2.</t>
+  </si>
+  <si>
+    <t>..a rough split granite monument, triangular in shape, marked A B L. and situated at a junction of walls, about one-half mile southwest of Fort pond and about 680 feet southeast of the West Acton road</t>
   </si>
   <si>
     <t>probably never placed: too close to corner</t>
@@ -736,7 +736,7 @@
     <t>Summer Street</t>
   </si>
   <si>
-    <t>Summer  Rd</t>
+    <t>Summer Rd</t>
   </si>
   <si>
     <t>south side, near boundary sign</t>
@@ -2266,15 +2266,15 @@
       </c>
       <c r="C3" s="4">
         <f>countifs(Monuments!$N$2:$N$52,$B3,Monuments!C$2:C$52,"X")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D3" s="4">
         <f>countifs(Monuments!$N$2:$N$52,$B3,Monuments!D$2:D$52,"X")</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" s="4">
         <f>countifs(Monuments!$N$2:$N$52,$B3,Monuments!E$2:E$52,"X")</f>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F3" s="4">
         <f>countifs(Monuments!$N$2:$N$52,$B3,Monuments!F$2:F$52,"X")</f>
@@ -2298,7 +2298,7 @@
       </c>
       <c r="K3" s="4">
         <f>countif(Monuments!N$2:N$52,B3)</f>
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="4">
@@ -2348,15 +2348,15 @@
       </c>
       <c r="C5" s="4">
         <f>countifs(Monuments!$N$2:$N$52,$B5,Monuments!C$2:C$52,"X")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D5" s="4">
         <f>countifs(Monuments!$N$2:$N$52,$B5,Monuments!D$2:D$52,"X")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E5" s="4">
         <f>countifs(Monuments!$N$2:$N$52,$B5,Monuments!E$2:E$52,"X")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F5" s="4">
         <f>countifs(Monuments!$N$2:$N$52,$B5,Monuments!F$2:F$52,"X")</f>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="K5" s="4">
         <f>countif(Monuments!N$2:N$52,B5)</f>
-        <v>15</v>
+        <v>17</v>
       </c>
     </row>
     <row r="6">
@@ -3937,7 +3937,7 @@
     <row r="20">
       <c r="A20" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Acton/Westford Bay  Drive (East)</v>
+        <v>Acton/Westford Bay Drive (East)</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>60</v>
@@ -4021,7 +4021,7 @@
         <v>153</v>
       </c>
       <c r="N21" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O21" s="20">
         <v>45580.0</v>
@@ -5149,7 +5149,7 @@
         <v>218</v>
       </c>
       <c r="N37" s="1" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="O37" s="20">
         <v>45792.0</v>
@@ -24470,8 +24470,8 @@
         <v>roadstone on the northeasterly side of Bear Hill road</v>
       </c>
       <c r="S18" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"looked where a private road crosses the boundary (but no bounds were found there). These coodinates are where that road crosses the border.")</f>
-        <v>looked where a private road crosses the boundary (but no bounds were found there). These coodinates are where that road crosses the border.</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"looked where a private road crosses the boundary (but no bounds were found there). These coordinates are where that road crosses the border.")</f>
+        <v>looked where a private road crosses the boundary (but no bounds were found there). These coordinates are where that road crosses the border.</v>
       </c>
       <c r="T18" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"map estimate ")</f>
@@ -24503,8 +24503,8 @@
       <c r="I19" s="5"/>
       <c r="J19" s="5"/>
       <c r="K19" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Bay  Drive (East)")</f>
-        <v>Bay  Drive (East)</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Bay Drive (East)")</f>
+        <v>Bay Drive (East)</v>
       </c>
       <c r="L19" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Street Crossing")</f>
@@ -24569,8 +24569,8 @@
         <v>Avalon</v>
       </c>
       <c r="O20" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Documented")</f>
-        <v>Documented</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Not Found")</f>
+        <v>Not Found</v>
       </c>
       <c r="P20" s="29">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),45580.0)</f>
@@ -24756,16 +24756,16 @@
         <v>45924</v>
       </c>
       <c r="Q23" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Visible from the southeast corner of the fenced in area behind the main barm of Bobby's Ranch")</f>
-        <v>Visible from the southeast corner of the fenced in area behind the main barm of Bobby's Ranch</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Visible from the southeast corner of the fenced in area behind the main barn of Bobby's Ranch")</f>
+        <v>Visible from the southeast corner of the fenced in area behind the main barn of Bobby's Ranch</v>
       </c>
       <c r="R23" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"a rough split granite monument, triangular In shape, marked A L W 1832, and situated in low woodland near an open meadow, about 800 feet northwest of a cart path leading northeasterly from Nagog pond and about 2,500 feet distant from the pond;")</f>
         <v>a rough split granite monument, triangular In shape, marked A L W 1832, and situated in low woodland near an open meadow, about 800 feet northwest of a cart path leading northeasterly from Nagog pond and about 2,500 feet distant from the pond;</v>
       </c>
       <c r="S23" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Contact owners at Bobby's Ranch before any visit. You need towalk through barn, and electricity to fence needs to be turned off.")</f>
-        <v>Contact owners at Bobby's Ranch before any visit. You need towalk through barn, and electricity to fence needs to be turned off.</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Contact owners at Bobby's Ranch before any visit. You need to walk through barn, and electricity to fence needs to be turned off.")</f>
+        <v>Contact owners at Bobby's Ranch before any visit. You need to walk through barn, and electricity to fence needs to be turned off.</v>
       </c>
       <c r="T23" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"State")</f>
@@ -24818,8 +24818,8 @@
         <v>45810</v>
       </c>
       <c r="Q24" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"same as Nashoba Road corner?")</f>
-        <v>same as Nashoba Road corner?</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Maybe never installed because it would have been so close to the Acton/Littleton monument?")</f>
+        <v>Maybe never installed because it would have been so close to the Acton/Littleton monument?</v>
       </c>
       <c r="R24" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"no")</f>
@@ -24881,8 +24881,8 @@
         <v>next to stone wall near end of Nashoba Road</v>
       </c>
       <c r="R25" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"corner 1, a rough split granite monument of irregular shape marked A L 1831 and situated at the northerly end of Nagog pond, on the northeasterly side of the road leading from North Acton to Littletown;")</f>
-        <v>corner 1, a rough split granite monument of irregular shape marked A L 1831 and situated at the northerly end of Nagog pond, on the northeasterly side of the road leading from North Acton to Littletown;</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"corner 1, a rough split granite monument of irregular shape marked A L 1831 and situated at the northerly end of Nagog pond, on the northeasterly side of the road leading from North Acton to Littletown[sic]")</f>
+        <v>corner 1, a rough split granite monument of irregular shape marked A L 1831 and situated at the northerly end of Nagog pond, on the northeasterly side of the road leading from North Acton to Littletown[sic]</v>
       </c>
       <c r="S25" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"lying on ground. Too difficult to paint. Will seek to get it rescued.")</f>
@@ -24939,8 +24939,8 @@
         <v>45810</v>
       </c>
       <c r="Q26" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"same as Nashoba Road corner?")</f>
-        <v>same as Nashoba Road corner?</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Maybe never installed because it would have been so close to the Acton/Littleton monument?")</f>
+        <v>Maybe never installed because it would have been so close to the Acton/Littleton monument?</v>
       </c>
       <c r="R26" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"no")</f>
@@ -24998,8 +24998,8 @@
         <v>45810</v>
       </c>
       <c r="Q27" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"near bottom of AWD land. roughly follow tree acros path near pond uphill")</f>
-        <v>near bottom of AWD land. roughly follow tree acros path near pond uphill</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"near bottom of AWD land. roughly follow tree across path near pond uphill")</f>
+        <v>near bottom of AWD land. roughly follow tree across path near pond uphill</v>
       </c>
       <c r="R27" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"corner 2, a rough split granite monument of irregular shape marked A L 1831, and situated in heavy maple, oak and chestnut woods, about 288 feet from the southwesterly shore of Nagog pond.")</f>
@@ -25461,24 +25461,24 @@
         <v>Newtown Road</v>
       </c>
       <c r="N35" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Rte 2 Exit 115 (Newtown/Central")</f>
-        <v>Rte 2 Exit 115 (Newtown/Central</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Rte 2 Exit 115 (Newtown/Central Street)")</f>
+        <v>Rte 2 Exit 115 (Newtown/Central Street)</v>
       </c>
       <c r="O35" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Documented")</f>
-        <v>Documented</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Not Found")</f>
+        <v>Not Found</v>
       </c>
       <c r="P35" s="29">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),45792.0)</f>
         <v>45792</v>
       </c>
       <c r="Q35" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"looked a couple of times, not found yet. Boxborough reports it is missing")</f>
-        <v>looked a couple of times, not found yet. Boxborough reports it is missing</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"looked a couple of times, not found yet. Boxborough reports it is missing. I think it would be in the grassy area between lanes of the exits. Unlikely to survive the construction of Rte 2.")</f>
+        <v>looked a couple of times, not found yet. Boxborough reports it is missing. I think it would be in the grassy area between lanes of the exits. Unlikely to survive the construction of Rte 2.</v>
       </c>
       <c r="R35" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"..a rough split granite monument, triangular in shape, marked A B L. and situated at a junction of walls, about one-half mile southwest of Fort pond and about 680 feet southeast of the West Acton road;")</f>
-        <v>..a rough split granite monument, triangular in shape, marked A B L. and situated at a junction of walls, about one-half mile southwest of Fort pond and about 680 feet southeast of the West Acton road;</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"..a rough split granite monument, triangular in shape, marked A B L. and situated at a junction of walls, about one-half mile southwest of Fort pond and about 680 feet southeast of the West Acton road")</f>
+        <v>..a rough split granite monument, triangular in shape, marked A B L. and situated at a junction of walls, about one-half mile southwest of Fort pond and about 680 feet southeast of the West Acton road</v>
       </c>
       <c r="S35" s="5"/>
       <c r="T35" s="5" t="str">
@@ -25749,8 +25749,8 @@
         <v>Street Crossing</v>
       </c>
       <c r="M40" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Summer  Rd")</f>
-        <v>Summer  Rd</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Summer Rd")</f>
+        <v>Summer Rd</v>
       </c>
       <c r="N40" s="5"/>
       <c r="O40" s="5" t="str">
@@ -32638,8 +32638,8 @@
     </row>
     <row r="20">
       <c r="A20" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Acton/Westford Bay  Drive (East)")</f>
-        <v>Acton/Westford Bay  Drive (East)</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Acton/Westford Bay Drive (East)")</f>
+        <v>Acton/Westford Bay Drive (East)</v>
       </c>
     </row>
     <row r="21">

</xml_diff>

<commit_message>
Add generate_geocoding_csv.py, export coords for Geoapify
lon/lat-only CSV per Jim's spec for Geoapify's drag-and-drop
reverse-geocoding tool. Also picks up Jim's latest coordinate/manifest
edits in the re-exported xlsx.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Acton Bounds.xlsx
+++ b/Acton Bounds.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="536">
   <si>
     <t>Count by status/town</t>
   </si>
@@ -702,7 +702,7 @@
     <t>-71.45672</t>
   </si>
   <si>
-    <t>Find maps of old path of road, and survey.</t>
+    <t xml:space="preserve">Find maps of old path of road, and look near old road crossing. Would have been added after 1904, or may be what the W B marker is pointing to. </t>
   </si>
   <si>
     <t>W B Marker on Fort Pond Road</t>
@@ -778,6 +778,9 @@
   </si>
   <si>
     <t>-71.453932</t>
+  </si>
+  <si>
+    <t>Get a picture of the Maynard side of the monument</t>
   </si>
   <si>
     <t>Parker Street</t>
@@ -984,7 +987,13 @@
     <t>linestone" known as Cat Head Rock between Acton - Westford 1 and the corner of Acton - Littleton - Westford.</t>
   </si>
   <si>
+    <t>Walk between ALW and AW1 looking for possible bear hill road</t>
+  </si>
+  <si>
     <t>Where Westford Lane gets to Westford. There is a corner behind a fence with many stones. Might be in there?</t>
+  </si>
+  <si>
+    <t>no, unless this is the same as Cat Head Rock from 1904.</t>
   </si>
   <si>
     <t>42.527574</t>
@@ -5513,6 +5522,9 @@
       <c r="AD39" s="21">
         <v>47.0</v>
       </c>
+      <c r="AE39" s="3" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="1" t="str">
@@ -5526,13 +5538,13 @@
         <v>53</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="N40" s="1" t="s">
         <v>13</v>
@@ -5541,19 +5553,19 @@
         <v>241</v>
       </c>
       <c r="P40" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="Q40" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="R40" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="S40" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T40" s="17" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="U40" s="5">
         <f t="shared" si="51"/>
@@ -5568,7 +5580,7 @@
         <v>32.2044</v>
       </c>
       <c r="X40" s="26" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="Y40" s="5">
         <f t="shared" si="54"/>
@@ -5590,7 +5602,7 @@
         <v>49.0</v>
       </c>
       <c r="AE40" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="41">
@@ -5609,7 +5621,7 @@
       </c>
       <c r="L41" s="1"/>
       <c r="M41" s="1" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="N41" s="1" t="s">
         <v>12</v>
@@ -5618,17 +5630,17 @@
         <v>45770.0</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="Q41" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="R41" s="4"/>
       <c r="S41" s="3" t="s">
         <v>69</v>
       </c>
       <c r="T41" s="17" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="U41" s="5">
         <f t="shared" si="51"/>
@@ -5643,7 +5655,7 @@
         <v>20.076</v>
       </c>
       <c r="X41" s="17" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Y41" s="5">
         <f t="shared" si="54"/>
@@ -5665,7 +5677,7 @@
         <v>50.0</v>
       </c>
       <c r="AE41" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
     </row>
     <row r="42">
@@ -5680,13 +5692,13 @@
         <v>53</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="N42" s="1" t="s">
         <v>12</v>
@@ -5695,17 +5707,17 @@
         <v>45862.0</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="Q42" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="R42" s="4"/>
       <c r="S42" s="3" t="s">
         <v>69</v>
       </c>
       <c r="T42" s="17" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="U42" s="5">
         <f t="shared" ref="U42:U43" si="57">abs(trunc(T42))</f>
@@ -5720,7 +5732,7 @@
         <v>13.7328</v>
       </c>
       <c r="X42" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Y42" s="5">
         <f t="shared" ref="Y42:Y50" si="60">abs(trunc(X42))</f>
@@ -5742,7 +5754,7 @@
         <v>51.0</v>
       </c>
       <c r="AE42" s="3" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
     </row>
     <row r="43">
@@ -5760,23 +5772,23 @@
         <v>53</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="L43" s="1"/>
       <c r="M43" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="N43" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O43" s="25" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="P43" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="Q43" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="R43" s="1"/>
       <c r="S43" s="3" t="s">
@@ -5832,7 +5844,7 @@
         <v>53</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="L44" s="1"/>
       <c r="M44" s="4"/>
@@ -5843,17 +5855,17 @@
         <v>241</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="R44" s="1"/>
       <c r="S44" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T44" s="17" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="U44" s="5">
         <f t="shared" ref="U44:U46" si="63">if(isblank(T44),"",abs(trunc(T44)))</f>
@@ -5868,7 +5880,7 @@
         <v>5.4108</v>
       </c>
       <c r="X44" s="17" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="Y44" s="5">
         <f t="shared" si="60"/>
@@ -5902,13 +5914,13 @@
         <v>53</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="N45" s="1" t="s">
         <v>13</v>
@@ -5917,17 +5929,17 @@
         <v>241</v>
       </c>
       <c r="P45" s="1" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="R45" s="1"/>
       <c r="S45" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T45" s="17" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="U45" s="5">
         <f t="shared" si="63"/>
@@ -5942,7 +5954,7 @@
         <v>12.204</v>
       </c>
       <c r="X45" s="17" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="Y45" s="5">
         <f t="shared" si="60"/>
@@ -5976,10 +5988,10 @@
         <v>53</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="M46" s="4"/>
       <c r="N46" s="1" t="s">
@@ -5989,17 +6001,17 @@
         <v>241</v>
       </c>
       <c r="P46" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="Q46" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="R46" s="1"/>
       <c r="S46" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T46" s="17" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="U46" s="5">
         <f t="shared" si="63"/>
@@ -6014,7 +6026,7 @@
         <v>34.8912</v>
       </c>
       <c r="X46" s="17" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="Y46" s="5">
         <f t="shared" si="60"/>
@@ -6048,11 +6060,11 @@
         <v>53</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="L47" s="1"/>
       <c r="M47" s="1" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="N47" s="1" t="s">
         <v>12</v>
@@ -6061,10 +6073,10 @@
         <v>45580.0</v>
       </c>
       <c r="P47" s="1" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="Q47" s="1" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="R47" s="1"/>
       <c r="S47" s="3" t="s">
@@ -6108,7 +6120,7 @@
         <v>20.0</v>
       </c>
       <c r="AE47" s="3" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
     </row>
     <row r="48">
@@ -6123,7 +6135,7 @@
         <v>53</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="L48" s="1"/>
       <c r="M48" s="4"/>
@@ -6134,7 +6146,7 @@
         <v>45580.0</v>
       </c>
       <c r="P48" s="1" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="Q48" s="1" t="s">
         <v>74</v>
@@ -6144,7 +6156,7 @@
         <v>69</v>
       </c>
       <c r="T48" s="17" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="U48" s="5">
         <f t="shared" si="66"/>
@@ -6159,7 +6171,7 @@
         <v>34.5144</v>
       </c>
       <c r="X48" s="17" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="Y48" s="5">
         <f t="shared" si="60"/>
@@ -6196,7 +6208,7 @@
         <v>53</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="L49" s="1"/>
       <c r="M49" s="4"/>
@@ -6207,7 +6219,7 @@
         <v>45580.0</v>
       </c>
       <c r="P49" s="1" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="Q49" s="1" t="s">
         <v>74</v>
@@ -6217,7 +6229,7 @@
         <v>69</v>
       </c>
       <c r="T49" s="17" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="U49" s="5">
         <f t="shared" si="66"/>
@@ -6232,7 +6244,7 @@
         <v>37.398</v>
       </c>
       <c r="X49" s="17" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="Y49" s="5">
         <f t="shared" si="60"/>
@@ -6266,7 +6278,7 @@
         <v>53</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="L50" s="1"/>
       <c r="M50" s="4"/>
@@ -6275,19 +6287,19 @@
       </c>
       <c r="O50" s="15"/>
       <c r="P50" s="1" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="Q50" s="1" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="R50" s="1" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="S50" s="3" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="T50" s="17" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="U50" s="5">
         <f t="shared" si="66"/>
@@ -6302,7 +6314,7 @@
         <v>51.042</v>
       </c>
       <c r="X50" s="17" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="Y50" s="5">
         <f t="shared" si="60"/>
@@ -6324,7 +6336,7 @@
         <v>18.0</v>
       </c>
       <c r="AE50" s="3" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
     </row>
     <row r="51">
@@ -6336,7 +6348,7 @@
         <v>52</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="K51" s="1" t="s">
         <v>111</v>
@@ -6348,10 +6360,10 @@
       </c>
       <c r="O51" s="15"/>
       <c r="P51" s="1" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="Q51" s="1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="R51" s="4"/>
       <c r="T51" s="17"/>
@@ -6367,6 +6379,9 @@
       <c r="AD51" s="21">
         <v>23.0</v>
       </c>
+      <c r="AE51" s="3" t="s">
+        <v>320</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="1" t="str">
@@ -6386,7 +6401,7 @@
         <v>234</v>
       </c>
       <c r="M52" s="1" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="N52" s="1" t="s">
         <v>12</v>
@@ -6395,17 +6410,17 @@
         <v>45580.0</v>
       </c>
       <c r="P52" s="1" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="Q52" s="1" t="s">
-        <v>74</v>
+        <v>322</v>
       </c>
       <c r="R52" s="4"/>
       <c r="S52" s="3" t="s">
         <v>69</v>
       </c>
       <c r="T52" s="17" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="U52" s="5">
         <f>abs(trunc(T52))</f>
@@ -6420,7 +6435,7 @@
         <v>39.2664</v>
       </c>
       <c r="X52" s="17" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="Y52" s="5">
         <f>abs(trunc(X52))</f>
@@ -6442,7 +6457,7 @@
         <v>22.0</v>
       </c>
       <c r="AE52" s="3" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
     </row>
     <row r="53">
@@ -21513,10 +21528,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="31" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B1" s="31" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="C1" s="32"/>
       <c r="D1" s="32"/>
@@ -21736,22 +21751,22 @@
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="38" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B12" s="38" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="D12" s="38" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="E12" s="39" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F12" s="39" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="G12" s="39" t="s">
         <v>179</v>
@@ -21760,206 +21775,206 @@
         <v>241</v>
       </c>
       <c r="I12" s="39" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="J12" s="39" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="K12" s="39" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="L12" s="39" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="M12" s="10"/>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="40" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="B13" s="40" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="C13" s="40" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="D13" s="41"/>
       <c r="E13" s="40" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F13" s="42" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="G13" s="42" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="H13" s="42" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="I13" s="42" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="J13" s="42" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="K13" s="42" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="L13" s="42" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="43" t="s">
+        <v>342</v>
+      </c>
+      <c r="B14" s="43" t="s">
+        <v>343</v>
+      </c>
+      <c r="C14" s="43" t="s">
         <v>339</v>
-      </c>
-      <c r="B14" s="43" t="s">
-        <v>340</v>
-      </c>
-      <c r="C14" s="43" t="s">
-        <v>336</v>
       </c>
       <c r="D14" s="44"/>
       <c r="E14" s="43" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F14" s="45" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="G14" s="45" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="H14" s="45" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="I14" s="45" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="J14" s="45" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="K14" s="45" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="L14" s="44"/>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="40" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B15" s="40" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="C15" s="40" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="D15" s="41"/>
       <c r="E15" s="40" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="F15" s="46" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="G15" s="46" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="H15" s="46" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="I15" s="46" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="J15" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="K15" s="46" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="L15" s="41"/>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="43" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B16" s="43" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="C16" s="43" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="D16" s="44"/>
       <c r="E16" s="43" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F16" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="G16" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="H16" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="I16" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="J16" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="K16" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="L16" s="44"/>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="40" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B17" s="40" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="C17" s="40" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="D17" s="41"/>
       <c r="E17" s="40" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F17" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="G17" s="46" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="H17" s="46" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="I17" s="46" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="J17" s="46" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="K17" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="L17" s="41"/>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="43" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B18" s="43" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="C18" s="43" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="D18" s="43" t="s">
         <v>2</v>
       </c>
       <c r="E18" s="43" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F18" s="44"/>
       <c r="G18" s="44"/>
@@ -21967,25 +21982,25 @@
       <c r="I18" s="44"/>
       <c r="J18" s="44"/>
       <c r="K18" s="45" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="L18" s="44"/>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="40" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B19" s="40" t="s">
+        <v>361</v>
+      </c>
+      <c r="C19" s="40" t="s">
         <v>358</v>
-      </c>
-      <c r="C19" s="40" t="s">
-        <v>355</v>
       </c>
       <c r="D19" s="40" t="s">
         <v>2</v>
       </c>
       <c r="E19" s="40" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F19" s="41"/>
       <c r="G19" s="41"/>
@@ -21993,25 +22008,25 @@
       <c r="I19" s="41"/>
       <c r="J19" s="41"/>
       <c r="K19" s="46" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="L19" s="41"/>
     </row>
     <row r="20" ht="22.5" customHeight="1">
       <c r="A20" s="43" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B20" s="43" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="C20" s="43" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="D20" s="43" t="s">
         <v>2</v>
       </c>
       <c r="E20" s="43" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="F20" s="44"/>
       <c r="G20" s="44"/>
@@ -22019,65 +22034,65 @@
       <c r="I20" s="44"/>
       <c r="J20" s="44"/>
       <c r="K20" s="45" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="L20" s="44"/>
     </row>
     <row r="21" ht="22.5" customHeight="1">
       <c r="A21" s="40" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B21" s="40" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="C21" s="40" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="D21" s="41"/>
       <c r="E21" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="F21" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="G21" s="46" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="H21" s="46" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="I21" s="47" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="J21" s="47" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="K21" s="47" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="L21" s="41"/>
     </row>
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="45" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="B22" s="45" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="C22" s="44"/>
       <c r="D22" s="45" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="E22" s="44"/>
       <c r="F22" s="44"/>
       <c r="G22" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="H22" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="I22" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="J22" s="44"/>
       <c r="K22" s="44"/>
@@ -22085,25 +22100,25 @@
     </row>
     <row r="23" ht="22.5" customHeight="1">
       <c r="A23" s="46" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="B23" s="46" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="C23" s="41"/>
       <c r="D23" s="46" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="E23" s="41"/>
       <c r="F23" s="41"/>
       <c r="G23" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="H23" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="I23" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="J23" s="41"/>
       <c r="K23" s="41"/>
@@ -22111,25 +22126,25 @@
     </row>
     <row r="24" ht="22.5" customHeight="1">
       <c r="A24" s="45" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B24" s="45" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="C24" s="44"/>
       <c r="D24" s="45" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="E24" s="44"/>
       <c r="F24" s="44"/>
       <c r="G24" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="H24" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="I24" s="48" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="J24" s="49"/>
       <c r="K24" s="49"/>
@@ -22137,10 +22152,10 @@
     </row>
     <row r="25" ht="22.5" customHeight="1">
       <c r="A25" s="46" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="B25" s="46" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="C25" s="41"/>
       <c r="D25" s="46" t="s">
@@ -22149,13 +22164,13 @@
       <c r="E25" s="41"/>
       <c r="F25" s="41"/>
       <c r="G25" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="H25" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="I25" s="47" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="J25" s="50"/>
       <c r="K25" s="50"/>
@@ -22163,13 +22178,13 @@
     </row>
     <row r="26" ht="22.5" customHeight="1">
       <c r="A26" s="45" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="B26" s="45" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="C26" s="44" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="D26" s="45" t="s">
         <v>6</v>
@@ -22177,11 +22192,11 @@
       <c r="E26" s="49"/>
       <c r="F26" s="44"/>
       <c r="G26" s="45" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="H26" s="44"/>
       <c r="I26" s="48" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="J26" s="44"/>
       <c r="K26" s="44"/>
@@ -22189,13 +22204,13 @@
     </row>
     <row r="27" ht="22.5" customHeight="1">
       <c r="A27" s="46" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="B27" s="46" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="C27" s="41" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="D27" s="46" t="s">
         <v>6</v>
@@ -22203,11 +22218,11 @@
       <c r="E27" s="50"/>
       <c r="F27" s="41"/>
       <c r="G27" s="46" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="H27" s="41"/>
       <c r="I27" s="47" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="J27" s="41"/>
       <c r="K27" s="41"/>
@@ -22215,10 +22230,10 @@
     </row>
     <row r="28" ht="22.5" customHeight="1">
       <c r="A28" s="45" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B28" s="45" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="C28" s="44"/>
       <c r="D28" s="45" t="s">
@@ -22227,26 +22242,26 @@
       <c r="E28" s="44"/>
       <c r="F28" s="44"/>
       <c r="G28" s="45" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="H28" s="45" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="I28" s="45" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="J28" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="K28" s="44"/>
       <c r="L28" s="44"/>
     </row>
     <row r="29" ht="22.5" customHeight="1">
       <c r="A29" s="46" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="B29" s="46" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="C29" s="41"/>
       <c r="D29" s="46" t="s">
@@ -22255,26 +22270,26 @@
       <c r="E29" s="41"/>
       <c r="F29" s="41"/>
       <c r="G29" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="H29" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="I29" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="J29" s="46" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="K29" s="41"/>
       <c r="L29" s="41"/>
     </row>
     <row r="30" ht="22.5" customHeight="1">
       <c r="A30" s="45" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="B30" s="45" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="C30" s="44"/>
       <c r="D30" s="45" t="s">
@@ -22283,26 +22298,26 @@
       <c r="E30" s="44"/>
       <c r="F30" s="44"/>
       <c r="G30" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="H30" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="I30" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="J30" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="K30" s="44"/>
       <c r="L30" s="44"/>
     </row>
     <row r="31" ht="22.5" customHeight="1">
       <c r="A31" s="46" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="B31" s="46" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="C31" s="41"/>
       <c r="D31" s="46" t="s">
@@ -22311,26 +22326,26 @@
       <c r="E31" s="41"/>
       <c r="F31" s="41"/>
       <c r="G31" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="H31" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="I31" s="46" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="J31" s="46" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="K31" s="41"/>
       <c r="L31" s="41"/>
     </row>
     <row r="32" ht="22.5" customHeight="1">
       <c r="A32" s="45" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="B32" s="45" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="C32" s="44"/>
       <c r="D32" s="45" t="s">
@@ -22339,23 +22354,23 @@
       <c r="E32" s="44"/>
       <c r="F32" s="44"/>
       <c r="G32" s="45" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="H32" s="45" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="I32" s="48" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="J32" s="48" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="K32" s="49"/>
       <c r="L32" s="44"/>
     </row>
     <row r="33" ht="22.5" customHeight="1">
       <c r="A33" s="46" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B33" s="41"/>
       <c r="C33" s="41"/>
@@ -22368,14 +22383,14 @@
       <c r="H33" s="41"/>
       <c r="I33" s="41"/>
       <c r="J33" s="46" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="K33" s="41"/>
       <c r="L33" s="41"/>
     </row>
     <row r="34" ht="22.5" customHeight="1">
       <c r="A34" s="45" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="B34" s="44"/>
       <c r="C34" s="44"/>
@@ -22388,17 +22403,17 @@
       <c r="H34" s="44"/>
       <c r="I34" s="44"/>
       <c r="J34" s="45" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="K34" s="44"/>
       <c r="L34" s="44"/>
     </row>
     <row r="35" ht="22.5" customHeight="1">
       <c r="A35" s="46" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B35" s="46" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="C35" s="41"/>
       <c r="D35" s="46" t="s">
@@ -22410,17 +22425,17 @@
       <c r="H35" s="41"/>
       <c r="I35" s="41"/>
       <c r="J35" s="46" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="K35" s="41"/>
       <c r="L35" s="41"/>
     </row>
     <row r="36" ht="22.5" customHeight="1">
       <c r="A36" s="45" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="B36" s="45" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="C36" s="44"/>
       <c r="D36" s="45" t="s">
@@ -22433,16 +22448,16 @@
       <c r="I36" s="44"/>
       <c r="J36" s="44"/>
       <c r="K36" s="45" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="L36" s="44"/>
     </row>
     <row r="37" ht="22.5" customHeight="1">
       <c r="A37" s="46" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
       <c r="B37" s="46" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="C37" s="41"/>
       <c r="D37" s="41"/>
@@ -22453,19 +22468,19 @@
       <c r="I37" s="41"/>
       <c r="J37" s="41"/>
       <c r="K37" s="46" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="L37" s="41"/>
     </row>
     <row r="38" ht="22.5" customHeight="1">
       <c r="A38" s="48" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
       <c r="B38" s="48" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="C38" s="51" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="D38" s="52" t="s">
         <v>8</v>
@@ -22475,11 +22490,11 @@
       <c r="G38" s="44"/>
       <c r="H38" s="44"/>
       <c r="I38" s="52" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="J38" s="49"/>
       <c r="K38" s="48" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="L38" s="44"/>
     </row>
@@ -22500,70 +22515,70 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>82</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
     </row>
     <row r="2">
@@ -22600,19 +22615,19 @@
         <v>-71.47352778</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="K2" s="3">
         <v>53.0</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="M2" s="53" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="Q2" s="3">
         <v>916626.0</v>
@@ -22621,10 +22636,10 @@
         <v>202175.0</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="U2" s="3">
         <v>546632.0</v>
@@ -22633,10 +22648,10 @@
         <v>607006.0</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="Y2" s="3">
         <v>-7956396.90869999</v>
@@ -22679,19 +22694,19 @@
         <v>-71.49854444</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="K3" s="3">
         <v>53.0</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="M3" s="53" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="Q3" s="3">
         <v>912582.0</v>
@@ -22700,10 +22715,10 @@
         <v>200119.0</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
       <c r="U3" s="3">
         <v>533365.0</v>
@@ -22712,10 +22727,10 @@
         <v>600259.0</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="Y3" s="3">
         <v>-7959181.92299999</v>
@@ -22758,19 +22773,19 @@
         <v>-71.39156111</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="K4" s="3">
         <v>53.0</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="M4" s="53" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="Q4" s="3">
         <v>917369.0</v>
@@ -22779,10 +22794,10 @@
         <v>208912.0</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="U4" s="3">
         <v>549070.0</v>
@@ -22791,10 +22806,10 @@
         <v>629107.0</v>
       </c>
       <c r="W4" s="3" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="X4" s="3" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="Y4" s="3">
         <v>-7947272.57209999</v>
@@ -22837,19 +22852,19 @@
         <v>-71.39794444</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="K5" s="3">
         <v>53.0</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="M5" s="53" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="Q5" s="3">
         <v>919537.0</v>
@@ -22858,10 +22873,10 @@
         <v>208385.0</v>
       </c>
       <c r="S5" s="3" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="U5" s="3">
         <v>556180.0</v>
@@ -22870,10 +22885,10 @@
         <v>627377.0</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="X5" s="3" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="Y5" s="3">
         <v>-7947983.11989999</v>
@@ -22916,19 +22931,19 @@
         <v>-71.38494444</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="K6" s="3">
         <v>53.0</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="M6" s="53" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="Q6" s="3">
         <v>917108.0</v>
@@ -22937,10 +22952,10 @@
         <v>209456.0</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="T6" s="3" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="U6" s="3">
         <v>548214.0</v>
@@ -22949,10 +22964,10 @@
         <v>630892.0</v>
       </c>
       <c r="W6" s="3" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="X6" s="3" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="Y6" s="3">
         <v>-7946536.00149999</v>
@@ -22995,19 +23010,19 @@
         <v>-71.39951389</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="K7" s="3">
         <v>53.0</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="M7" s="53" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="Q7" s="3">
         <v>920390.0</v>
@@ -23016,10 +23031,10 @@
         <v>208255.0</v>
       </c>
       <c r="S7" s="3" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="T7" s="3" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="U7" s="3">
         <v>558979.0</v>
@@ -23028,10 +23043,10 @@
         <v>626951.0</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="X7" s="3" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="Y7" s="3">
         <v>-7948157.69009999</v>
@@ -23074,19 +23089,19 @@
         <v>-71.43039167</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="K8" s="3">
         <v>53.0</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="M8" s="53" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="Q8" s="3">
         <v>909604.0</v>
@@ -23095,10 +23110,10 @@
         <v>205727.0</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="U8" s="3">
         <v>523592.0</v>
@@ -23107,10 +23122,10 @@
         <v>618657.0</v>
       </c>
       <c r="W8" s="3" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="X8" s="3" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="Y8" s="3">
         <v>-7951595.17399999</v>
@@ -23153,19 +23168,19 @@
         <v>-71.43501667</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="K9" s="3">
         <v>53.0</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="M9" s="53" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="Q9" s="3">
         <v>919071.0</v>
@@ -23174,10 +23189,10 @@
         <v>205339.0</v>
       </c>
       <c r="S9" s="3" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="T9" s="3" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="U9" s="3">
         <v>554653.0</v>
@@ -23186,10 +23201,10 @@
         <v>617385.0</v>
       </c>
       <c r="W9" s="3" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="X9" s="3" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="Y9" s="3">
         <v>-7952109.8181</v>
@@ -23232,19 +23247,19 @@
         <v>-71.44393889</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="K10" s="3">
         <v>53.0</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="M10" s="53" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="Q10" s="3">
         <v>917614.0</v>
@@ -23253,10 +23268,10 @@
         <v>204607.0</v>
       </c>
       <c r="S10" s="3" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="T10" s="3" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="U10" s="3">
         <v>549873.0</v>
@@ -23265,10 +23280,10 @@
         <v>614983.0</v>
       </c>
       <c r="W10" s="3" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="X10" s="3" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="Y10" s="3">
         <v>-7953103.0547</v>
@@ -23311,19 +23326,19 @@
         <v>-71.42853333</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="K11" s="3">
         <v>53.0</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="M11" s="53" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="Q11" s="3">
         <v>919808.0</v>
@@ -23332,10 +23347,10 @@
         <v>205871.0</v>
       </c>
       <c r="S11" s="3" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="T11" s="3" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="U11" s="3">
         <v>557071.0</v>
@@ -23344,10 +23359,10 @@
         <v>619131.0</v>
       </c>
       <c r="W11" s="3" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="X11" s="3" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="Y11" s="3">
         <v>-7951388.09019999</v>
@@ -23390,19 +23405,19 @@
         <v>-71.46432778</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="K12" s="3">
         <v>53.0</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="M12" s="53" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="Q12" s="3">
         <v>911088.0</v>
@@ -23411,10 +23426,10 @@
         <v>202934.0</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="T12" s="3" t="s">
-        <v>485</v>
+        <v>488</v>
       </c>
       <c r="U12" s="3">
         <v>528463.0</v>
@@ -23423,10 +23438,10 @@
         <v>609494.0</v>
       </c>
       <c r="W12" s="3" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="X12" s="3" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="Y12" s="3">
         <v>-7955372.7137</v>
@@ -23469,19 +23484,19 @@
         <v>-71.42379444</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="K13" s="3">
         <v>53.0</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="M13" s="53" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="Q13" s="3">
         <v>919518.0</v>
@@ -23490,10 +23505,10 @@
         <v>206261.0</v>
       </c>
       <c r="S13" s="3" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="T13" s="3" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="U13" s="3">
         <v>556120.0</v>
@@ -23502,10 +23517,10 @@
         <v>620409.0</v>
       </c>
       <c r="W13" s="3" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="X13" s="3" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="Y13" s="3">
         <v>-7950860.55109999</v>
@@ -23625,7 +23640,7 @@
         <v>Coordinate Source</v>
       </c>
       <c r="U1" s="6" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="V1" s="37"/>
       <c r="W1" s="37"/>
@@ -26503,8 +26518,8 @@
         <v>Where Westford Lane gets to Westford. There is a corner behind a fence with many stones. Might be in there?</v>
       </c>
       <c r="R50" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"no")</f>
-        <v>no</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"no, unless this is the same as Cat Head Rock from 1904.")</f>
+        <v>no, unless this is the same as Cat Head Rock from 1904.</v>
       </c>
       <c r="S50" s="5"/>
       <c r="T50" s="5" t="str">
@@ -26596,13 +26611,13 @@
         <v>Longitude</v>
       </c>
       <c r="P1" s="6" t="s">
-        <v>495</v>
+        <v>498</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="S1" s="37"/>
       <c r="T1" s="37"/>
@@ -33014,24 +33029,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="60" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="B1" s="60" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="C1" s="60" t="s">
-        <v>500</v>
+        <v>503</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="B2" s="5" t="str">
         <f t="array" ref="B2">index($G$14:BO$14,0,MATCH(MIN(ABS(G2:R2)), ABS(G2:R2),0))</f>
@@ -33100,7 +33115,7 @@
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="B3" s="5" t="str">
         <f t="array" ref="B3">index($G$14:BO$14,0,MATCH(MIN(ABS(G3:R3)), ABS(G3:R3),0))</f>
@@ -33169,7 +33184,7 @@
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="B4" s="5" t="str">
         <f t="array" ref="B4">index($G$14:BO$14,0,MATCH(MIN(ABS(G4:R4)), ABS(G4:R4),0))</f>
@@ -33238,7 +33253,7 @@
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="B5" s="5" t="str">
         <f t="array" ref="B5">index($G$14:BO$14,0,MATCH(MIN(ABS(G5:R5)), ABS(G5:R5),0))</f>
@@ -33307,7 +33322,7 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="B6" s="5" t="str">
         <f t="array" ref="B6">index($G$14:BO$14,0,MATCH(MIN(ABS(G6:R6)), ABS(G6:R6),0))</f>
@@ -33376,7 +33391,7 @@
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="B7" s="5" t="str">
         <f t="array" ref="B7">index($G$14:BO$14,0,MATCH(MIN(ABS(G7:R7)), ABS(G7:R7),0))</f>
@@ -33445,7 +33460,7 @@
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B8" s="5" t="str">
         <f t="array" ref="B8">index($G$14:BO$14,0,MATCH(MIN(ABS(G8:R8)), ABS(G8:R8),0))</f>
@@ -33514,7 +33529,7 @@
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="B9" s="5" t="str">
         <f t="array" ref="B9">index($G$14:BO$14,0,MATCH(MIN(ABS(G9:R9)), ABS(G9:R9),0))</f>
@@ -33583,7 +33598,7 @@
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="B10" s="5" t="str">
         <f t="array" ref="B10">index($G$14:BO$14,0,MATCH(MIN(ABS(G10:R10)), ABS(G10:R10),0))</f>
@@ -33652,7 +33667,7 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="B11" s="5" t="str">
         <f t="array" ref="B11">index($G$14:BO$14,0,MATCH(MIN(ABS(G11:R11)), ABS(G11:R11),0))</f>
@@ -33721,7 +33736,7 @@
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B12" s="5" t="str">
         <f t="array" ref="B12">index($G$14:BO$14,0,MATCH(MIN(ABS(G12:R12)), ABS(G12:R12),0))</f>
@@ -33790,7 +33805,7 @@
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="B13" s="5" t="str">
         <f t="array" ref="B13">index($G$14:BO$14,0,MATCH(MIN(ABS(G13:R13)), ABS(G13:R13),0))</f>
@@ -33863,7 +33878,7 @@
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
       <c r="F14" s="3" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="G14" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("transpose(filter(Monuments!A$2:A918,Monuments!B2:B918=""Corner""))"),"Acton/Boxborough/Littleton")</f>
@@ -33920,7 +33935,7 @@
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
       <c r="F15" s="3" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="G15" s="3">
         <f>IFERROR(__xludf.DUMMYFUNCTION("transpose(filter(Monuments!X$2:X918,Monuments!B2:B918=""Corner""))"),-71.473529496)</f>
@@ -33977,7 +33992,7 @@
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
       <c r="F16" s="3" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="G16" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("transpose(filter(Monuments!T$2:T918,Monuments!B2:B918=""Corner""))"),42.5001860150001)</f>
@@ -34030,7 +34045,7 @@
     </row>
     <row r="17">
       <c r="F17" s="3" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="G17" s="5" t="str">
         <f t="shared" ref="G17:R17" si="15">vlookup(G$14,$B:$E,4,False)</f>
@@ -34083,7 +34098,7 @@
     </row>
     <row r="18">
       <c r="F18" s="3" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="G18" s="5" t="str">
         <f t="shared" ref="G18:R18" si="16">vlookup(G$14,$B:$E,3,False)</f>
@@ -34136,7 +34151,7 @@
     </row>
     <row r="19">
       <c r="F19" s="3" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="G19" s="62">
         <f t="shared" ref="G19:R19" si="17">G17-G15</f>
@@ -34189,7 +34204,7 @@
     </row>
     <row r="20">
       <c r="F20" s="3" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="G20" s="62">
         <f t="shared" ref="G20:R20" si="18">G18-G16</f>
@@ -34268,7 +34283,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="B2" s="3">
         <v>42.5001860150001</v>
@@ -34279,7 +34294,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B3" s="3">
         <v>42.4637837510001</v>
@@ -34290,7 +34305,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="B4" s="3">
         <v>42.5068287080001</v>
@@ -34301,7 +34316,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="B5" s="3">
         <v>42.526344807</v>
@@ -34312,7 +34327,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="B6" s="3">
         <v>42.504473137</v>
@@ -34323,7 +34338,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="B7" s="3">
         <v>42.534025086</v>
@@ -34334,7 +34349,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>527</v>
+        <v>530</v>
       </c>
       <c r="B8" s="3">
         <v>42.436947994</v>
@@ -34345,7 +34360,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="B9" s="3">
         <v>42.5221791480001</v>
@@ -34356,7 +34371,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="B10" s="3">
         <v>42.509068563</v>
@@ -34367,7 +34382,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="B11" s="3">
         <v>42.528812154</v>
@@ -34378,7 +34393,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="B12" s="3">
         <v>42.4503286410001</v>
@@ -34389,7 +34404,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="B13" s="3">
         <v>42.5261982760001</v>

</xml_diff>

<commit_message>
Re-export Acton Bounds.xlsx: Type=Witness for the two witness monuments
Monuments!B13 (Acton/Carlisle/Concord witness) Corner -> Witness and
Monuments!B36 (Fort Pond Road W B Marker) Street Crossing -> Witness,
matching the Witness icon the overview map uses. Remaining diff cells are
cached-value cascades in helper sheets (For Mapping/For Measuring/
SiteNames/OpenStreetMap) from the re-export, not independent edits.
Contacts sheet unchanged; no Email/Phone/personal data changed.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Acton Bounds.xlsx
+++ b/Acton Bounds.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="536">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="537">
   <si>
     <t>Count by status/town</t>
   </si>
@@ -367,6 +367,9 @@
   </si>
   <si>
     <t>Survey at edge of Ben's Woods</t>
+  </si>
+  <si>
+    <t>Witness</t>
   </si>
   <si>
     <t>Pope Road</t>
@@ -3543,7 +3546,7 @@
         <v>Acton/Carlisle/Concord</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>82</v>
+        <v>115</v>
       </c>
       <c r="F13" s="3" t="s">
         <v>53</v>
@@ -3552,11 +3555,11 @@
         <v>53</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="N13" s="1" t="s">
         <v>13</v>
@@ -3565,13 +3568,13 @@
         <v>45838.0</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="R13" s="1" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="S13" s="3" t="s">
         <v>69</v>
@@ -3633,7 +3636,7 @@
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="N14" s="1" t="s">
         <v>13</v>
@@ -3642,10 +3645,10 @@
         <v>45838.0</v>
       </c>
       <c r="P14" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="Q14" s="16" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="R14" s="1"/>
       <c r="S14" s="3" t="s">
@@ -3701,11 +3704,11 @@
         <v>53</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="L15" s="1"/>
       <c r="M15" s="1" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="N15" s="1" t="s">
         <v>13</v>
@@ -3715,16 +3718,16 @@
       </c>
       <c r="P15" s="4"/>
       <c r="Q15" s="16" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="R15" s="1" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="S15" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T15" s="17" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="U15" s="5">
         <f t="shared" ref="U15:U20" si="24">if(isblank(T15),"",abs(trunc(T15)))</f>
@@ -3739,7 +3742,7 @@
         <v>24.114</v>
       </c>
       <c r="X15" s="24" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="Y15" s="5">
         <f t="shared" si="21"/>
@@ -3773,13 +3776,13 @@
         <v>53</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="M16" s="1" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="N16" s="1" t="s">
         <v>11</v>
@@ -3788,19 +3791,19 @@
         <v>45989.0</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q16" s="1" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="R16" s="1" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="S16" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T16" s="25" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="U16" s="5">
         <f t="shared" si="24"/>
@@ -3815,7 +3818,7 @@
         <v>20.334</v>
       </c>
       <c r="X16" s="17" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Y16" s="5">
         <f t="shared" si="21"/>
@@ -3837,7 +3840,7 @@
         <v>7.0</v>
       </c>
       <c r="AE16" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="17">
@@ -3852,7 +3855,7 @@
         <v>53</v>
       </c>
       <c r="K17" s="1" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="L17" s="1"/>
       <c r="M17" s="4"/>
@@ -3863,7 +3866,7 @@
         <v>45770.0</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="Q17" s="1" t="s">
         <v>74</v>
@@ -3873,7 +3876,7 @@
         <v>69</v>
       </c>
       <c r="T17" s="17" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="U17" s="5">
         <f t="shared" si="24"/>
@@ -3888,7 +3891,7 @@
         <v>31.9272</v>
       </c>
       <c r="X17" s="17" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Y17" s="5">
         <f t="shared" si="21"/>
@@ -3910,7 +3913,7 @@
         <v>3.0</v>
       </c>
       <c r="AE17" s="3" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
     <row r="18">
@@ -3925,7 +3928,7 @@
         <v>53</v>
       </c>
       <c r="K18" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="L18" s="1"/>
       <c r="M18" s="4"/>
@@ -3936,17 +3939,17 @@
         <v>45838.0</v>
       </c>
       <c r="P18" s="1" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Q18" s="1" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="R18" s="4"/>
       <c r="S18" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T18" s="17" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="U18" s="5">
         <f t="shared" si="24"/>
@@ -3961,7 +3964,7 @@
         <v>35.4924</v>
       </c>
       <c r="X18" s="17" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="Y18" s="5">
         <f t="shared" ref="Y18:Y20" si="27">if(isblank(X18),"",abs(trunc(X18)))</f>
@@ -3995,11 +3998,11 @@
         <v>53</v>
       </c>
       <c r="K19" s="1" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="L19" s="1"/>
       <c r="M19" s="1" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="N19" s="1" t="s">
         <v>13</v>
@@ -4008,17 +4011,17 @@
         <v>45924.0</v>
       </c>
       <c r="P19" s="1" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="Q19" s="1" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="R19" s="1"/>
       <c r="S19" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T19" s="25" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="U19" s="5">
         <f t="shared" si="24"/>
@@ -4033,7 +4036,7 @@
         <v>24.6564</v>
       </c>
       <c r="X19" s="17" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="Y19" s="5">
         <f t="shared" si="27"/>
@@ -4067,11 +4070,11 @@
         <v>53</v>
       </c>
       <c r="K20" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="L20" s="1"/>
       <c r="M20" s="1" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="N20" s="1" t="s">
         <v>13</v>
@@ -4081,14 +4084,14 @@
       </c>
       <c r="P20" s="1"/>
       <c r="Q20" s="16" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="R20" s="4"/>
       <c r="S20" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T20" s="17" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="U20" s="5">
         <f t="shared" si="24"/>
@@ -4103,7 +4106,7 @@
         <v>11.9376</v>
       </c>
       <c r="X20" s="17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="Y20" s="5">
         <f t="shared" si="27"/>
@@ -4137,7 +4140,7 @@
         <v>53</v>
       </c>
       <c r="K21" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="L21" s="1"/>
       <c r="M21" s="4"/>
@@ -4148,17 +4151,17 @@
         <v>45770.0</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="Q21" s="1" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="R21" s="4"/>
       <c r="S21" s="3" t="s">
         <v>69</v>
       </c>
       <c r="T21" s="17" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="U21" s="5">
         <f>abs(trunc(T21))</f>
@@ -4173,7 +4176,7 @@
         <v>30.75</v>
       </c>
       <c r="X21" s="17" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="Y21" s="5">
         <f t="shared" ref="Y21:Y27" si="30">abs(trunc(X21))</f>
@@ -4195,7 +4198,7 @@
         <v>2.0</v>
       </c>
       <c r="AE21" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
     </row>
     <row r="22">
@@ -4214,7 +4217,7 @@
       </c>
       <c r="L22" s="1"/>
       <c r="M22" s="1" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="N22" s="1" t="s">
         <v>12</v>
@@ -4223,7 +4226,7 @@
         <v>45405.0</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="Q22" s="1" t="s">
         <v>68</v>
@@ -4233,7 +4236,7 @@
         <v>69</v>
       </c>
       <c r="T22" s="17" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="U22" s="5">
         <f t="shared" ref="U22:U24" si="33">if(isblank(T22),"",abs(trunc(T22)))</f>
@@ -4248,7 +4251,7 @@
         <v>9.3144</v>
       </c>
       <c r="X22" s="17" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="Y22" s="5">
         <f t="shared" si="30"/>
@@ -4270,7 +4273,7 @@
         <v>6.0</v>
       </c>
       <c r="AE22" s="3" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="23">
@@ -4285,7 +4288,7 @@
         <v>53</v>
       </c>
       <c r="K23" s="1" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="L23" s="1"/>
       <c r="M23" s="4"/>
@@ -4296,17 +4299,17 @@
         <v>45838.0</v>
       </c>
       <c r="P23" s="1" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="Q23" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="R23" s="1"/>
       <c r="S23" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T23" s="17" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="U23" s="5">
         <f t="shared" si="33"/>
@@ -4321,7 +4324,7 @@
         <v>8.3268</v>
       </c>
       <c r="X23" s="17" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="Y23" s="5">
         <f t="shared" si="30"/>
@@ -4355,7 +4358,7 @@
         <v>53</v>
       </c>
       <c r="K24" s="1" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="L24" s="1"/>
       <c r="M24" s="4"/>
@@ -4367,14 +4370,14 @@
       </c>
       <c r="P24" s="4"/>
       <c r="Q24" s="16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="R24" s="4"/>
       <c r="S24" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T24" s="17" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="U24" s="5">
         <f t="shared" si="33"/>
@@ -4389,7 +4392,7 @@
         <v>28.4388</v>
       </c>
       <c r="X24" s="17" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="Y24" s="5">
         <f t="shared" si="30"/>
@@ -4429,26 +4432,26 @@
         <v>53</v>
       </c>
       <c r="K25" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="L25" s="1"/>
       <c r="M25" s="1" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="N25" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O25" s="26" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="P25" s="1" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="Q25" s="1" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="R25" s="1" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="S25" s="3" t="s">
         <v>87</v>
@@ -4503,26 +4506,26 @@
         <v>53</v>
       </c>
       <c r="K26" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="L26" s="1"/>
       <c r="M26" s="1" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="N26" s="1" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="O26" s="15">
         <v>45810.0</v>
       </c>
       <c r="P26" s="1" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="Q26" s="16" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="R26" s="1" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="S26" s="3" t="s">
         <v>87</v>
@@ -4568,7 +4571,7 @@
         <v>26.0</v>
       </c>
       <c r="AE26" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
     </row>
     <row r="27">
@@ -4583,11 +4586,11 @@
         <v>53</v>
       </c>
       <c r="K27" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="L27" s="1"/>
       <c r="M27" s="1" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="N27" s="1" t="s">
         <v>13</v>
@@ -4596,10 +4599,10 @@
         <v>45810.0</v>
       </c>
       <c r="P27" s="1" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="Q27" s="16" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="R27" s="1"/>
       <c r="S27" s="3" t="s">
@@ -4658,10 +4661,10 @@
         <v>53</v>
       </c>
       <c r="K28" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="L28" s="1" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="M28" s="4"/>
       <c r="N28" s="1" t="s">
@@ -4671,7 +4674,7 @@
         <v>45741.0</v>
       </c>
       <c r="P28" s="1" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="Q28" s="1" t="s">
         <v>74</v>
@@ -4681,7 +4684,7 @@
         <v>69</v>
       </c>
       <c r="T28" s="17" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="U28" s="5">
         <f t="shared" si="36"/>
@@ -4696,7 +4699,7 @@
         <v>8.496</v>
       </c>
       <c r="X28" s="17" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="Y28" s="5">
         <f t="shared" ref="Y28:Y29" si="39">if(isblank(X28),"",abs(trunc(X28)))</f>
@@ -4718,7 +4721,7 @@
         <v>33.0</v>
       </c>
       <c r="AE28" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="29">
@@ -4733,10 +4736,10 @@
         <v>53</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="L29" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="M29" s="1"/>
       <c r="N29" s="1" t="s">
@@ -4747,14 +4750,14 @@
       </c>
       <c r="P29" s="1"/>
       <c r="Q29" s="16" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="R29" s="1"/>
       <c r="S29" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T29" s="24" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="U29" s="5">
         <f t="shared" si="36"/>
@@ -4769,7 +4772,7 @@
         <v>21.5496</v>
       </c>
       <c r="X29" s="24" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Y29" s="5">
         <f t="shared" si="39"/>
@@ -4803,10 +4806,10 @@
         <v>53</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="L30" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="M30" s="4"/>
       <c r="N30" s="1" t="s">
@@ -4816,7 +4819,7 @@
         <v>45810.0</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Q30" s="1" t="s">
         <v>74</v>
@@ -4826,7 +4829,7 @@
         <v>69</v>
       </c>
       <c r="T30" s="17" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="U30" s="5">
         <f t="shared" si="36"/>
@@ -4841,7 +4844,7 @@
         <v>21.072</v>
       </c>
       <c r="X30" s="17" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="Y30" s="5">
         <f>abs(trunc(X30))</f>
@@ -4875,10 +4878,10 @@
         <v>53</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="M31" s="4"/>
       <c r="N31" s="1" t="s">
@@ -4888,7 +4891,7 @@
         <v>45741.0</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="Q31" s="1" t="s">
         <v>74</v>
@@ -4898,7 +4901,7 @@
         <v>69</v>
       </c>
       <c r="T31" s="17" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="U31" s="5">
         <f>if(isblank(T31),"",abs(trunc(T31)))</f>
@@ -4913,7 +4916,7 @@
         <v>4.0788</v>
       </c>
       <c r="X31" s="17" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="Y31" s="5">
         <f>if(isblank(X31),"",abs(trunc(X31)))</f>
@@ -4935,7 +4938,7 @@
         <v>35.0</v>
       </c>
       <c r="AE31" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="32">
@@ -4950,10 +4953,10 @@
         <v>53</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="L32" s="1" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="M32" s="4"/>
       <c r="N32" s="1" t="s">
@@ -4963,16 +4966,16 @@
         <v>45810.0</v>
       </c>
       <c r="P32" s="1" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="Q32" s="16" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="S32" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T32" s="24" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="U32" s="5">
         <f t="shared" ref="U32:U37" si="42">abs(trunc(T32))</f>
@@ -4987,7 +4990,7 @@
         <v>26.7372</v>
       </c>
       <c r="X32" s="24" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="Y32" s="5">
         <f t="shared" ref="Y32:Y33" si="45">abs(trunc(X32))</f>
@@ -5021,10 +5024,10 @@
         <v>53</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="L33" s="1" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="M33" s="4"/>
       <c r="N33" s="1" t="s">
@@ -5034,7 +5037,7 @@
         <v>45810.0</v>
       </c>
       <c r="P33" s="1" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Q33" s="1" t="s">
         <v>74</v>
@@ -5044,7 +5047,7 @@
         <v>69</v>
       </c>
       <c r="T33" s="17" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="U33" s="5">
         <f t="shared" si="42"/>
@@ -5059,7 +5062,7 @@
         <v>19.74</v>
       </c>
       <c r="X33" s="17" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="Y33" s="5">
         <f t="shared" si="45"/>
@@ -5096,10 +5099,10 @@
         <v>83</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="N34" s="1" t="s">
         <v>13</v>
@@ -5109,14 +5112,14 @@
       </c>
       <c r="P34" s="1"/>
       <c r="Q34" s="16" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="R34" s="4"/>
       <c r="S34" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T34" s="17" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="U34" s="5">
         <f t="shared" si="42"/>
@@ -5131,7 +5134,7 @@
         <v>5.1012</v>
       </c>
       <c r="X34" s="17" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="Y34" s="5">
         <f t="shared" ref="Y34:Y36" si="48">if(isblank(X34),"",abs(trunc(X34)))</f>
@@ -5165,7 +5168,7 @@
         <v>53</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="L35" s="1"/>
       <c r="M35" s="4"/>
@@ -5176,7 +5179,7 @@
         <v>45810.0</v>
       </c>
       <c r="P35" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="Q35" s="1" t="s">
         <v>74</v>
@@ -5186,7 +5189,7 @@
         <v>69</v>
       </c>
       <c r="T35" s="17" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="U35" s="5">
         <f t="shared" si="42"/>
@@ -5201,7 +5204,7 @@
         <v>18.972</v>
       </c>
       <c r="X35" s="17" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="Y35" s="5">
         <f t="shared" si="48"/>
@@ -5223,25 +5226,25 @@
         <v>32.0</v>
       </c>
       <c r="AE35" s="3" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>Acton/Littleton W B Marker on Fort Pond Road</v>
+        <v>Acton/Littleton</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>52</v>
+        <v>115</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>53</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="L36" s="1" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="M36" s="1"/>
       <c r="N36" s="1" t="s">
@@ -5251,19 +5254,19 @@
         <v>45810.0</v>
       </c>
       <c r="P36" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="Q36" s="16" t="s">
         <v>74</v>
       </c>
       <c r="R36" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="S36" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T36" s="24" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="U36" s="5">
         <f t="shared" si="42"/>
@@ -5278,7 +5281,7 @@
         <v>22.3236</v>
       </c>
       <c r="X36" s="24" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="Y36" s="5">
         <f t="shared" si="48"/>
@@ -5300,7 +5303,7 @@
         <v>31.0</v>
       </c>
       <c r="AE36" s="3" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="37">
@@ -5318,13 +5321,13 @@
         <v>53</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="N37" s="1" t="s">
         <v>13</v>
@@ -5333,13 +5336,13 @@
         <v>45924.0</v>
       </c>
       <c r="P37" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="Q37" s="16" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="R37" s="1" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="S37" s="3" t="s">
         <v>87</v>
@@ -5394,30 +5397,30 @@
         <v>53</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L38" s="1"/>
       <c r="M38" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="N38" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O38" s="26" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="P38" s="1" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="Q38" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="R38" s="1"/>
       <c r="S38" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T38" s="24" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="U38" s="5">
         <f t="shared" ref="U38:U41" si="51">if(isblank(T38),"",abs(trunc(T38)))</f>
@@ -5432,7 +5435,7 @@
         <v>44.5236</v>
       </c>
       <c r="X38" s="27" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="Y38" s="5">
         <f t="shared" ref="Y38:Y41" si="54">if(isblank(X38),"",abs(trunc(X38)))</f>
@@ -5469,29 +5472,29 @@
         <v>103</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="N39" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O39" s="26" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="P39" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="Q39" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="R39" s="1"/>
       <c r="S39" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T39" s="28" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="U39" s="5">
         <f t="shared" si="51"/>
@@ -5506,7 +5509,7 @@
         <v>46.428</v>
       </c>
       <c r="X39" s="27" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="Y39" s="5">
         <f t="shared" si="54"/>
@@ -5528,7 +5531,7 @@
         <v>47.0</v>
       </c>
       <c r="AE39" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
     </row>
     <row r="40">
@@ -5543,34 +5546,34 @@
         <v>53</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="N40" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O40" s="26" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="P40" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="Q40" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="R40" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="S40" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T40" s="17" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="U40" s="5">
         <f t="shared" si="51"/>
@@ -5585,7 +5588,7 @@
         <v>32.2044</v>
       </c>
       <c r="X40" s="27" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="Y40" s="5">
         <f t="shared" si="54"/>
@@ -5607,7 +5610,7 @@
         <v>49.0</v>
       </c>
       <c r="AE40" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
     </row>
     <row r="41">
@@ -5622,11 +5625,11 @@
         <v>53</v>
       </c>
       <c r="K41" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="L41" s="1"/>
       <c r="M41" s="1" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="N41" s="1" t="s">
         <v>12</v>
@@ -5635,17 +5638,17 @@
         <v>45770.0</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="Q41" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="R41" s="4"/>
       <c r="S41" s="3" t="s">
         <v>69</v>
       </c>
       <c r="T41" s="17" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="U41" s="5">
         <f t="shared" si="51"/>
@@ -5660,7 +5663,7 @@
         <v>20.076</v>
       </c>
       <c r="X41" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="Y41" s="5">
         <f t="shared" si="54"/>
@@ -5682,7 +5685,7 @@
         <v>50.0</v>
       </c>
       <c r="AE41" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
     </row>
     <row r="42">
@@ -5697,13 +5700,13 @@
         <v>53</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="N42" s="1" t="s">
         <v>12</v>
@@ -5712,17 +5715,17 @@
         <v>45862.0</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="Q42" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="R42" s="4"/>
       <c r="S42" s="3" t="s">
         <v>69</v>
       </c>
       <c r="T42" s="17" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="U42" s="5">
         <f t="shared" ref="U42:U43" si="57">abs(trunc(T42))</f>
@@ -5737,7 +5740,7 @@
         <v>13.7328</v>
       </c>
       <c r="X42" s="17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="Y42" s="5">
         <f t="shared" ref="Y42:Y50" si="60">abs(trunc(X42))</f>
@@ -5759,7 +5762,7 @@
         <v>51.0</v>
       </c>
       <c r="AE42" s="3" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="43">
@@ -5777,23 +5780,23 @@
         <v>53</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="L43" s="1"/>
       <c r="M43" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="N43" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O43" s="26" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="P43" s="1" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="Q43" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="R43" s="1"/>
       <c r="S43" s="3" t="s">
@@ -5849,7 +5852,7 @@
         <v>53</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="L44" s="1"/>
       <c r="M44" s="4"/>
@@ -5857,20 +5860,20 @@
         <v>13</v>
       </c>
       <c r="O44" s="26" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="R44" s="1"/>
       <c r="S44" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T44" s="17" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="U44" s="5">
         <f t="shared" ref="U44:U46" si="63">if(isblank(T44),"",abs(trunc(T44)))</f>
@@ -5885,7 +5888,7 @@
         <v>5.4108</v>
       </c>
       <c r="X44" s="17" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="Y44" s="5">
         <f t="shared" si="60"/>
@@ -5919,32 +5922,32 @@
         <v>53</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="N45" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O45" s="26" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="P45" s="1" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="R45" s="1"/>
       <c r="S45" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T45" s="17" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="U45" s="5">
         <f t="shared" si="63"/>
@@ -5959,7 +5962,7 @@
         <v>12.204</v>
       </c>
       <c r="X45" s="17" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="Y45" s="5">
         <f t="shared" si="60"/>
@@ -5993,30 +5996,30 @@
         <v>53</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="M46" s="4"/>
       <c r="N46" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O46" s="26" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="P46" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="Q46" s="1" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="R46" s="1"/>
       <c r="S46" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T46" s="17" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="U46" s="5">
         <f t="shared" si="63"/>
@@ -6031,7 +6034,7 @@
         <v>34.8912</v>
       </c>
       <c r="X46" s="17" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="Y46" s="5">
         <f t="shared" si="60"/>
@@ -6065,11 +6068,11 @@
         <v>53</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="L47" s="1"/>
       <c r="M47" s="1" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="N47" s="1" t="s">
         <v>12</v>
@@ -6078,10 +6081,10 @@
         <v>45580.0</v>
       </c>
       <c r="P47" s="1" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="Q47" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="R47" s="1"/>
       <c r="S47" s="3" t="s">
@@ -6125,7 +6128,7 @@
         <v>20.0</v>
       </c>
       <c r="AE47" s="3" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
     </row>
     <row r="48">
@@ -6140,7 +6143,7 @@
         <v>53</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="L48" s="1"/>
       <c r="M48" s="4"/>
@@ -6151,7 +6154,7 @@
         <v>45580.0</v>
       </c>
       <c r="P48" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="Q48" s="1" t="s">
         <v>74</v>
@@ -6161,7 +6164,7 @@
         <v>69</v>
       </c>
       <c r="T48" s="17" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="U48" s="5">
         <f t="shared" si="66"/>
@@ -6176,7 +6179,7 @@
         <v>34.5144</v>
       </c>
       <c r="X48" s="17" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="Y48" s="5">
         <f t="shared" si="60"/>
@@ -6198,7 +6201,7 @@
         <v>19.0</v>
       </c>
       <c r="AE48" s="3" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="49">
@@ -6213,7 +6216,7 @@
         <v>53</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="L49" s="1"/>
       <c r="M49" s="4"/>
@@ -6224,7 +6227,7 @@
         <v>45580.0</v>
       </c>
       <c r="P49" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="Q49" s="1" t="s">
         <v>74</v>
@@ -6234,7 +6237,7 @@
         <v>69</v>
       </c>
       <c r="T49" s="17" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="U49" s="5">
         <f t="shared" si="66"/>
@@ -6249,7 +6252,7 @@
         <v>37.398</v>
       </c>
       <c r="X49" s="17" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="Y49" s="5">
         <f t="shared" si="60"/>
@@ -6283,7 +6286,7 @@
         <v>53</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="L50" s="1"/>
       <c r="M50" s="4"/>
@@ -6292,19 +6295,19 @@
       </c>
       <c r="O50" s="15"/>
       <c r="P50" s="1" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="Q50" s="1" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="R50" s="1" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="S50" s="3" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="T50" s="17" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="U50" s="5">
         <f t="shared" si="66"/>
@@ -6319,7 +6322,7 @@
         <v>51.042</v>
       </c>
       <c r="X50" s="17" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="Y50" s="5">
         <f t="shared" si="60"/>
@@ -6341,7 +6344,7 @@
         <v>18.0</v>
       </c>
       <c r="AE50" s="3" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
     </row>
     <row r="51">
@@ -6353,7 +6356,7 @@
         <v>52</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="K51" s="1" t="s">
         <v>111</v>
@@ -6365,10 +6368,10 @@
       </c>
       <c r="O51" s="15"/>
       <c r="P51" s="1" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="Q51" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="R51" s="4"/>
       <c r="T51" s="17"/>
@@ -6385,7 +6388,7 @@
         <v>23.0</v>
       </c>
       <c r="AE51" s="3" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
     </row>
     <row r="52">
@@ -6400,13 +6403,13 @@
         <v>53</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="M52" s="1" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="N52" s="1" t="s">
         <v>12</v>
@@ -6415,17 +6418,17 @@
         <v>45580.0</v>
       </c>
       <c r="P52" s="1" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="Q52" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="R52" s="4"/>
       <c r="S52" s="3" t="s">
         <v>69</v>
       </c>
       <c r="T52" s="17" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="U52" s="5">
         <f>abs(trunc(T52))</f>
@@ -6440,7 +6443,7 @@
         <v>39.2664</v>
       </c>
       <c r="X52" s="17" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="Y52" s="5">
         <f>abs(trunc(X52))</f>
@@ -6462,7 +6465,7 @@
         <v>22.0</v>
       </c>
       <c r="AE52" s="3" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
     </row>
     <row r="53">
@@ -21508,7 +21511,7 @@
       <formula1>"Painted,Found,Documented,Not Found,Unknown,Couldn't paint"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B52">
-      <formula1>"Corner,Street Crossing"</formula1>
+      <formula1>"Corner,Street Crossing,Witness"</formula1>
     </dataValidation>
   </dataValidations>
   <printOptions gridLines="1" horizontalCentered="1"/>
@@ -21533,10 +21536,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="32" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="B1" s="32" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="C1" s="33"/>
       <c r="D1" s="33"/>
@@ -21756,230 +21759,230 @@
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="39" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="B12" s="39" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="C12" s="39" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="D12" s="39" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="E12" s="40" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="F12" s="40" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="G12" s="40" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H12" s="40" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="I12" s="40" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="J12" s="40" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="K12" s="40" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="L12" s="40" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="M12" s="10"/>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="41" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="B13" s="41" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D13" s="42"/>
       <c r="E13" s="41" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F13" s="43" t="s">
+        <v>342</v>
+      </c>
+      <c r="G13" s="43" t="s">
+        <v>342</v>
+      </c>
+      <c r="H13" s="43" t="s">
+        <v>342</v>
+      </c>
+      <c r="I13" s="43" t="s">
+        <v>342</v>
+      </c>
+      <c r="J13" s="43" t="s">
+        <v>342</v>
+      </c>
+      <c r="K13" s="43" t="s">
+        <v>342</v>
+      </c>
+      <c r="L13" s="43" t="s">
         <v>341</v>
-      </c>
-      <c r="G13" s="43" t="s">
-        <v>341</v>
-      </c>
-      <c r="H13" s="43" t="s">
-        <v>341</v>
-      </c>
-      <c r="I13" s="43" t="s">
-        <v>341</v>
-      </c>
-      <c r="J13" s="43" t="s">
-        <v>341</v>
-      </c>
-      <c r="K13" s="43" t="s">
-        <v>341</v>
-      </c>
-      <c r="L13" s="43" t="s">
-        <v>340</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="44" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="C14" s="44" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="D14" s="45"/>
       <c r="E14" s="44" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F14" s="46" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G14" s="46" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="H14" s="46" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="I14" s="46" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J14" s="46" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K14" s="46" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="L14" s="45"/>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="41" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="B15" s="41" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="D15" s="42"/>
       <c r="E15" s="41" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F15" s="47" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="G15" s="47" t="s">
+        <v>349</v>
+      </c>
+      <c r="H15" s="47" t="s">
+        <v>349</v>
+      </c>
+      <c r="I15" s="47" t="s">
+        <v>349</v>
+      </c>
+      <c r="J15" s="47" t="s">
         <v>348</v>
       </c>
-      <c r="H15" s="47" t="s">
-        <v>348</v>
-      </c>
-      <c r="I15" s="47" t="s">
-        <v>348</v>
-      </c>
-      <c r="J15" s="47" t="s">
-        <v>347</v>
-      </c>
       <c r="K15" s="47" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L15" s="42"/>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="44" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="C16" s="44" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D16" s="45"/>
       <c r="E16" s="44" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F16" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="G16" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="H16" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="I16" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J16" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K16" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L16" s="45"/>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="41" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="B17" s="41" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="D17" s="42"/>
       <c r="E17" s="41" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F17" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G17" s="47" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="H17" s="47" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="I17" s="47" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J17" s="47" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K17" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="L17" s="42"/>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="44" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B18" s="44" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C18" s="44" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D18" s="44" t="s">
         <v>2</v>
       </c>
       <c r="E18" s="44" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F18" s="45"/>
       <c r="G18" s="45"/>
@@ -21987,25 +21990,25 @@
       <c r="I18" s="45"/>
       <c r="J18" s="45"/>
       <c r="K18" s="46" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="L18" s="45"/>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="41" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="B19" s="41" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="D19" s="41" t="s">
         <v>2</v>
       </c>
       <c r="E19" s="41" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F19" s="42"/>
       <c r="G19" s="42"/>
@@ -22013,25 +22016,25 @@
       <c r="I19" s="42"/>
       <c r="J19" s="42"/>
       <c r="K19" s="47" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L19" s="42"/>
     </row>
     <row r="20" ht="22.5" customHeight="1">
       <c r="A20" s="44" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="B20" s="44" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="C20" s="44" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="D20" s="44" t="s">
         <v>2</v>
       </c>
       <c r="E20" s="44" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="F20" s="45"/>
       <c r="G20" s="45"/>
@@ -22039,65 +22042,65 @@
       <c r="I20" s="45"/>
       <c r="J20" s="45"/>
       <c r="K20" s="46" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="L20" s="45"/>
     </row>
     <row r="21" ht="22.5" customHeight="1">
       <c r="A21" s="41" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="B21" s="41" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C21" s="41" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="D21" s="42"/>
       <c r="E21" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="F21" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="G21" s="47" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="H21" s="47" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="I21" s="48" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="J21" s="48" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="K21" s="48" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="L21" s="42"/>
     </row>
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="46" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="B22" s="46" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="C22" s="45"/>
       <c r="D22" s="46" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E22" s="45"/>
       <c r="F22" s="45"/>
       <c r="G22" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="H22" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="I22" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J22" s="45"/>
       <c r="K22" s="45"/>
@@ -22105,25 +22108,25 @@
     </row>
     <row r="23" ht="22.5" customHeight="1">
       <c r="A23" s="47" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="B23" s="47" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="C23" s="42"/>
       <c r="D23" s="47" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E23" s="42"/>
       <c r="F23" s="42"/>
       <c r="G23" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="H23" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="I23" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J23" s="42"/>
       <c r="K23" s="42"/>
@@ -22131,25 +22134,25 @@
     </row>
     <row r="24" ht="22.5" customHeight="1">
       <c r="A24" s="46" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="B24" s="46" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="C24" s="45"/>
       <c r="D24" s="46" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E24" s="45"/>
       <c r="F24" s="45"/>
       <c r="G24" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="H24" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="I24" s="49" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J24" s="50"/>
       <c r="K24" s="50"/>
@@ -22157,10 +22160,10 @@
     </row>
     <row r="25" ht="22.5" customHeight="1">
       <c r="A25" s="47" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="B25" s="47" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="C25" s="42"/>
       <c r="D25" s="47" t="s">
@@ -22169,13 +22172,13 @@
       <c r="E25" s="42"/>
       <c r="F25" s="42"/>
       <c r="G25" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="H25" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="I25" s="48" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J25" s="51"/>
       <c r="K25" s="51"/>
@@ -22183,13 +22186,13 @@
     </row>
     <row r="26" ht="22.5" customHeight="1">
       <c r="A26" s="46" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="B26" s="46" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="C26" s="45" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="D26" s="46" t="s">
         <v>6</v>
@@ -22197,11 +22200,11 @@
       <c r="E26" s="50"/>
       <c r="F26" s="45"/>
       <c r="G26" s="46" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="H26" s="45"/>
       <c r="I26" s="49" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J26" s="45"/>
       <c r="K26" s="45"/>
@@ -22209,13 +22212,13 @@
     </row>
     <row r="27" ht="22.5" customHeight="1">
       <c r="A27" s="47" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="B27" s="47" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="C27" s="42" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="D27" s="47" t="s">
         <v>6</v>
@@ -22223,11 +22226,11 @@
       <c r="E27" s="51"/>
       <c r="F27" s="42"/>
       <c r="G27" s="47" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="H27" s="42"/>
       <c r="I27" s="48" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J27" s="42"/>
       <c r="K27" s="42"/>
@@ -22235,10 +22238,10 @@
     </row>
     <row r="28" ht="22.5" customHeight="1">
       <c r="A28" s="46" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="B28" s="46" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="C28" s="45"/>
       <c r="D28" s="46" t="s">
@@ -22247,26 +22250,26 @@
       <c r="E28" s="45"/>
       <c r="F28" s="45"/>
       <c r="G28" s="46" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="H28" s="46" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="I28" s="46" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J28" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K28" s="45"/>
       <c r="L28" s="45"/>
     </row>
     <row r="29" ht="22.5" customHeight="1">
       <c r="A29" s="47" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="B29" s="47" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="C29" s="42"/>
       <c r="D29" s="47" t="s">
@@ -22275,26 +22278,26 @@
       <c r="E29" s="42"/>
       <c r="F29" s="42"/>
       <c r="G29" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="H29" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="I29" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J29" s="47" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K29" s="42"/>
       <c r="L29" s="42"/>
     </row>
     <row r="30" ht="22.5" customHeight="1">
       <c r="A30" s="46" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="B30" s="46" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="C30" s="45"/>
       <c r="D30" s="46" t="s">
@@ -22303,26 +22306,26 @@
       <c r="E30" s="45"/>
       <c r="F30" s="45"/>
       <c r="G30" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="H30" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="I30" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J30" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K30" s="45"/>
       <c r="L30" s="45"/>
     </row>
     <row r="31" ht="22.5" customHeight="1">
       <c r="A31" s="47" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="B31" s="47" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="C31" s="42"/>
       <c r="D31" s="47" t="s">
@@ -22331,26 +22334,26 @@
       <c r="E31" s="42"/>
       <c r="F31" s="42"/>
       <c r="G31" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="H31" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="I31" s="47" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J31" s="47" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K31" s="42"/>
       <c r="L31" s="42"/>
     </row>
     <row r="32" ht="22.5" customHeight="1">
       <c r="A32" s="46" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="B32" s="46" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="C32" s="45"/>
       <c r="D32" s="46" t="s">
@@ -22359,23 +22362,23 @@
       <c r="E32" s="45"/>
       <c r="F32" s="45"/>
       <c r="G32" s="46" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="H32" s="46" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="I32" s="49" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="J32" s="49" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K32" s="50"/>
       <c r="L32" s="45"/>
     </row>
     <row r="33" ht="22.5" customHeight="1">
       <c r="A33" s="47" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B33" s="42"/>
       <c r="C33" s="42"/>
@@ -22388,14 +22391,14 @@
       <c r="H33" s="42"/>
       <c r="I33" s="42"/>
       <c r="J33" s="47" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="K33" s="42"/>
       <c r="L33" s="42"/>
     </row>
     <row r="34" ht="22.5" customHeight="1">
       <c r="A34" s="46" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="B34" s="45"/>
       <c r="C34" s="45"/>
@@ -22408,17 +22411,17 @@
       <c r="H34" s="45"/>
       <c r="I34" s="45"/>
       <c r="J34" s="46" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="K34" s="45"/>
       <c r="L34" s="45"/>
     </row>
     <row r="35" ht="22.5" customHeight="1">
       <c r="A35" s="47" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B35" s="47" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C35" s="42"/>
       <c r="D35" s="47" t="s">
@@ -22430,17 +22433,17 @@
       <c r="H35" s="42"/>
       <c r="I35" s="42"/>
       <c r="J35" s="47" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="K35" s="42"/>
       <c r="L35" s="42"/>
     </row>
     <row r="36" ht="22.5" customHeight="1">
       <c r="A36" s="46" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="B36" s="46" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="C36" s="45"/>
       <c r="D36" s="46" t="s">
@@ -22453,16 +22456,16 @@
       <c r="I36" s="45"/>
       <c r="J36" s="45"/>
       <c r="K36" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L36" s="45"/>
     </row>
     <row r="37" ht="22.5" customHeight="1">
       <c r="A37" s="47" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="B37" s="47" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C37" s="42"/>
       <c r="D37" s="42"/>
@@ -22473,19 +22476,19 @@
       <c r="I37" s="42"/>
       <c r="J37" s="42"/>
       <c r="K37" s="47" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L37" s="42"/>
     </row>
     <row r="38" ht="22.5" customHeight="1">
       <c r="A38" s="49" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="B38" s="49" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C38" s="52" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="D38" s="53" t="s">
         <v>8</v>
@@ -22495,11 +22498,11 @@
       <c r="G38" s="45"/>
       <c r="H38" s="45"/>
       <c r="I38" s="53" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="J38" s="50"/>
       <c r="K38" s="49" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L38" s="45"/>
     </row>
@@ -22520,70 +22523,70 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>82</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
     </row>
     <row r="2">
@@ -22620,19 +22623,19 @@
         <v>-71.47352778</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="K2" s="3">
         <v>53.0</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M2" s="54" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="Q2" s="3">
         <v>916626.0</v>
@@ -22641,10 +22644,10 @@
         <v>202175.0</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="U2" s="3">
         <v>546632.0</v>
@@ -22653,10 +22656,10 @@
         <v>607006.0</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="Y2" s="3">
         <v>-7956396.90869999</v>
@@ -22699,19 +22702,19 @@
         <v>-71.49854444</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="K3" s="3">
         <v>53.0</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M3" s="54" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="Q3" s="3">
         <v>912582.0</v>
@@ -22720,10 +22723,10 @@
         <v>200119.0</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="U3" s="3">
         <v>533365.0</v>
@@ -22732,10 +22735,10 @@
         <v>600259.0</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="Y3" s="3">
         <v>-7959181.92299999</v>
@@ -22778,19 +22781,19 @@
         <v>-71.39156111</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="K4" s="3">
         <v>53.0</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M4" s="54" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="Q4" s="3">
         <v>917369.0</v>
@@ -22799,10 +22802,10 @@
         <v>208912.0</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="U4" s="3">
         <v>549070.0</v>
@@ -22811,10 +22814,10 @@
         <v>629107.0</v>
       </c>
       <c r="W4" s="3" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="X4" s="3" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="Y4" s="3">
         <v>-7947272.57209999</v>
@@ -22857,19 +22860,19 @@
         <v>-71.39794444</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="K5" s="3">
         <v>53.0</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M5" s="54" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="Q5" s="3">
         <v>919537.0</v>
@@ -22878,10 +22881,10 @@
         <v>208385.0</v>
       </c>
       <c r="S5" s="3" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="U5" s="3">
         <v>556180.0</v>
@@ -22890,10 +22893,10 @@
         <v>627377.0</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="X5" s="3" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="Y5" s="3">
         <v>-7947983.11989999</v>
@@ -22936,19 +22939,19 @@
         <v>-71.38494444</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="K6" s="3">
         <v>53.0</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M6" s="54" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="Q6" s="3">
         <v>917108.0</v>
@@ -22957,10 +22960,10 @@
         <v>209456.0</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="T6" s="3" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="U6" s="3">
         <v>548214.0</v>
@@ -22969,10 +22972,10 @@
         <v>630892.0</v>
       </c>
       <c r="W6" s="3" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="X6" s="3" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="Y6" s="3">
         <v>-7946536.00149999</v>
@@ -23015,19 +23018,19 @@
         <v>-71.39951389</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="K7" s="3">
         <v>53.0</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M7" s="54" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="Q7" s="3">
         <v>920390.0</v>
@@ -23036,10 +23039,10 @@
         <v>208255.0</v>
       </c>
       <c r="S7" s="3" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="T7" s="3" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="U7" s="3">
         <v>558979.0</v>
@@ -23048,10 +23051,10 @@
         <v>626951.0</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="X7" s="3" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="Y7" s="3">
         <v>-7948157.69009999</v>
@@ -23094,19 +23097,19 @@
         <v>-71.43039167</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="K8" s="3">
         <v>53.0</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M8" s="54" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="Q8" s="3">
         <v>909604.0</v>
@@ -23115,10 +23118,10 @@
         <v>205727.0</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="U8" s="3">
         <v>523592.0</v>
@@ -23127,10 +23130,10 @@
         <v>618657.0</v>
       </c>
       <c r="W8" s="3" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="X8" s="3" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="Y8" s="3">
         <v>-7951595.17399999</v>
@@ -23173,19 +23176,19 @@
         <v>-71.43501667</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="K9" s="3">
         <v>53.0</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M9" s="54" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="Q9" s="3">
         <v>919071.0</v>
@@ -23194,10 +23197,10 @@
         <v>205339.0</v>
       </c>
       <c r="S9" s="3" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="T9" s="3" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="U9" s="3">
         <v>554653.0</v>
@@ -23206,10 +23209,10 @@
         <v>617385.0</v>
       </c>
       <c r="W9" s="3" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="X9" s="3" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="Y9" s="3">
         <v>-7952109.8181</v>
@@ -23252,19 +23255,19 @@
         <v>-71.44393889</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="K10" s="3">
         <v>53.0</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M10" s="54" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="Q10" s="3">
         <v>917614.0</v>
@@ -23273,10 +23276,10 @@
         <v>204607.0</v>
       </c>
       <c r="S10" s="3" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="T10" s="3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="U10" s="3">
         <v>549873.0</v>
@@ -23285,10 +23288,10 @@
         <v>614983.0</v>
       </c>
       <c r="W10" s="3" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="X10" s="3" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="Y10" s="3">
         <v>-7953103.0547</v>
@@ -23331,19 +23334,19 @@
         <v>-71.42853333</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="K11" s="3">
         <v>53.0</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M11" s="54" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="Q11" s="3">
         <v>919808.0</v>
@@ -23352,10 +23355,10 @@
         <v>205871.0</v>
       </c>
       <c r="S11" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="T11" s="3" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="U11" s="3">
         <v>557071.0</v>
@@ -23364,10 +23367,10 @@
         <v>619131.0</v>
       </c>
       <c r="W11" s="3" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="X11" s="3" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="Y11" s="3">
         <v>-7951388.09019999</v>
@@ -23410,19 +23413,19 @@
         <v>-71.46432778</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="K12" s="3">
         <v>53.0</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M12" s="54" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="Q12" s="3">
         <v>911088.0</v>
@@ -23431,10 +23434,10 @@
         <v>202934.0</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="T12" s="3" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="U12" s="3">
         <v>528463.0</v>
@@ -23443,10 +23446,10 @@
         <v>609494.0</v>
       </c>
       <c r="W12" s="3" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="X12" s="3" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="Y12" s="3">
         <v>-7955372.7137</v>
@@ -23489,19 +23492,19 @@
         <v>-71.42379444</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="K13" s="3">
         <v>53.0</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="M13" s="54" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="Q13" s="3">
         <v>919518.0</v>
@@ -23510,10 +23513,10 @@
         <v>206261.0</v>
       </c>
       <c r="S13" s="3" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="T13" s="3" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="U13" s="3">
         <v>556120.0</v>
@@ -23522,10 +23525,10 @@
         <v>620409.0</v>
       </c>
       <c r="W13" s="3" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="X13" s="3" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="Y13" s="3">
         <v>-7950860.55109999</v>
@@ -23645,7 +23648,7 @@
         <v>Coordinate Source</v>
       </c>
       <c r="U1" s="6" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="V1" s="38"/>
       <c r="W1" s="38"/>
@@ -24280,8 +24283,8 @@
         <v>Pope Road</v>
       </c>
       <c r="L12" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Corner")</f>
-        <v>Corner</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Witness")</f>
+        <v>Witness</v>
       </c>
       <c r="M12" s="5"/>
       <c r="N12" s="5" t="str">
@@ -25631,8 +25634,8 @@
         <v>W B Marker on Fort Pond Road</v>
       </c>
       <c r="L35" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Street Crossing")</f>
-        <v>Street Crossing</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Witness")</f>
+        <v>Witness</v>
       </c>
       <c r="M35" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Fort Pond Road")</f>
@@ -26616,13 +26619,13 @@
         <v>Longitude</v>
       </c>
       <c r="P1" s="6" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="S1" s="38"/>
       <c r="T1" s="38"/>
@@ -26928,8 +26931,8 @@
         <v>Pope Road</v>
       </c>
       <c r="J9" s="59" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Corner")</f>
-        <v>Corner</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Witness")</f>
+        <v>Witness</v>
       </c>
       <c r="K9" s="60" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"394 Pope Road")</f>
@@ -27496,8 +27499,8 @@
         <v>W B Marker on Fort Pond Road</v>
       </c>
       <c r="J23" s="59" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Street Crossing")</f>
-        <v>Street Crossing</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Witness")</f>
+        <v>Witness</v>
       </c>
       <c r="K23" s="60"/>
       <c r="L23" s="59" t="str">
@@ -32917,8 +32920,8 @@
     </row>
     <row r="36">
       <c r="A36" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Acton/Littleton W B Marker on Fort Pond Road")</f>
-        <v>Acton/Littleton W B Marker on Fort Pond Road</v>
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Acton/Littleton")</f>
+        <v>Acton/Littleton</v>
       </c>
     </row>
     <row r="37">
@@ -33034,24 +33037,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="61" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="B1" s="61" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="C1" s="61" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="B2" s="5" t="str">
         <f t="array" ref="B2">index($G$14:BO$14,0,MATCH(MIN(ABS(G2:R2)), ABS(G2:R2),0))</f>
@@ -33087,40 +33090,40 @@
       </c>
       <c r="K2" s="62">
         <f t="shared" si="1"/>
-        <v>0.009165595831</v>
+        <v>0.01120558885</v>
       </c>
       <c r="L2" s="62">
         <f t="shared" si="1"/>
-        <v>0.01120558885</v>
+        <v>0.001330676926</v>
       </c>
       <c r="M2" s="62">
         <f t="shared" si="1"/>
-        <v>0.001330676926</v>
+        <v>0.006021331776</v>
       </c>
       <c r="N2" s="62">
         <f t="shared" si="1"/>
-        <v>0.006021331776</v>
+        <v>0.003865824739</v>
       </c>
       <c r="O2" s="62">
         <f t="shared" si="1"/>
-        <v>0.003865824739</v>
+        <v>0.007440579715</v>
       </c>
       <c r="P2" s="62">
         <f t="shared" si="1"/>
-        <v>0.007440579715</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="62">
         <f t="shared" si="1"/>
-        <v>0</v>
+        <v>0.007398852777</v>
       </c>
       <c r="R2" s="62">
         <f t="shared" si="1"/>
-        <v>0.007398852777</v>
+        <v>6909.181007</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B3" s="5" t="str">
         <f t="array" ref="B3">index($G$14:BO$14,0,MATCH(MIN(ABS(G3:R3)), ABS(G3:R3),0))</f>
@@ -33156,40 +33159,40 @@
       </c>
       <c r="K3" s="62">
         <f t="shared" si="4"/>
-        <v>0.01448795931</v>
+        <v>0.01474170363</v>
       </c>
       <c r="L3" s="62">
         <f t="shared" si="4"/>
-        <v>0.01474170363</v>
+        <v>0.005365400359</v>
       </c>
       <c r="M3" s="62">
         <f t="shared" si="4"/>
-        <v>0.005365400359</v>
+        <v>0.007446325415</v>
       </c>
       <c r="N3" s="62">
         <f t="shared" si="4"/>
-        <v>0.007446325415</v>
+        <v>0.005032919978</v>
       </c>
       <c r="O3" s="62">
         <f t="shared" si="4"/>
-        <v>0.005032919978</v>
+        <v>0.00913083408</v>
       </c>
       <c r="P3" s="62">
         <f t="shared" si="4"/>
-        <v>0.00913083408</v>
+        <v>0.001352171477</v>
       </c>
       <c r="Q3" s="62">
         <f t="shared" si="4"/>
-        <v>0.001352171477</v>
+        <v>0.009483781984</v>
       </c>
       <c r="R3" s="62">
         <f t="shared" si="4"/>
-        <v>0.009483781984</v>
+        <v>6915.215718</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B4" s="5" t="str">
         <f t="array" ref="B4">index($G$14:BO$14,0,MATCH(MIN(ABS(G4:R4)), ABS(G4:R4),0))</f>
@@ -33225,40 +33228,40 @@
       </c>
       <c r="K4" s="62">
         <f t="shared" si="5"/>
-        <v>0.006563895468</v>
+        <v>0.01037758307</v>
       </c>
       <c r="L4" s="62">
         <f t="shared" si="5"/>
-        <v>0.01037758307</v>
+        <v>0</v>
       </c>
       <c r="M4" s="62">
         <f t="shared" si="5"/>
-        <v>0</v>
+        <v>0.007285589844</v>
       </c>
       <c r="N4" s="62">
         <f t="shared" si="5"/>
-        <v>0.007285589844</v>
+        <v>0.005384683034</v>
       </c>
       <c r="O4" s="62">
         <f t="shared" si="5"/>
-        <v>0.005384683034</v>
+        <v>0.008442385134</v>
       </c>
       <c r="P4" s="62">
         <f t="shared" si="5"/>
-        <v>0.008442385134</v>
+        <v>0.001330337987</v>
       </c>
       <c r="Q4" s="62">
         <f t="shared" si="5"/>
-        <v>0.001330337987</v>
+        <v>0.008009097012</v>
       </c>
       <c r="R4" s="62">
         <f t="shared" si="5"/>
-        <v>0.008009097012</v>
+        <v>6903.196365</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B5" s="5" t="str">
         <f t="array" ref="B5">index($G$14:BO$14,0,MATCH(MIN(ABS(G5:R5)), ABS(G5:R5),0))</f>
@@ -33294,44 +33297,44 @@
       </c>
       <c r="K5" s="62">
         <f t="shared" si="6"/>
-        <v>0.007825252228</v>
+        <v>0.00662366547</v>
       </c>
       <c r="L5" s="62">
         <f t="shared" si="6"/>
-        <v>0.00662366547</v>
+        <v>0.005858488905</v>
       </c>
       <c r="M5" s="62">
         <f t="shared" si="6"/>
-        <v>0.005858488905</v>
+        <v>0.001967170272</v>
       </c>
       <c r="N5" s="62">
         <f t="shared" si="6"/>
-        <v>0.001967170272</v>
+        <v>0.0009545337125</v>
       </c>
       <c r="O5" s="62">
         <f t="shared" si="6"/>
-        <v>0.0009545337125</v>
+        <v>0.002844440636</v>
       </c>
       <c r="P5" s="62">
         <f t="shared" si="6"/>
-        <v>0.002844440636</v>
+        <v>0.002569525198</v>
       </c>
       <c r="Q5" s="62">
         <f t="shared" si="6"/>
-        <v>0.002569525198</v>
+        <v>0.003150487348</v>
       </c>
       <c r="R5" s="62">
         <f t="shared" si="6"/>
-        <v>0.003150487348</v>
+        <v>6914.73039</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B6" s="5" t="str">
         <f t="array" ref="B6">index($G$14:BO$14,0,MATCH(MIN(ABS(G6:R6)), ABS(G6:R6),0))</f>
-        <v>Acton/Carlisle/Concord</v>
+        <v>Acton/Carlisle 1</v>
       </c>
       <c r="C6" s="5" t="str">
         <f t="shared" si="2"/>
@@ -33363,40 +33366,40 @@
       </c>
       <c r="K6" s="62">
         <f t="shared" si="7"/>
-        <v>0.00000013789346</v>
+        <v>0.001086067572</v>
       </c>
       <c r="L6" s="62">
         <f t="shared" si="7"/>
-        <v>0.001086067572</v>
+        <v>0.006623988288</v>
       </c>
       <c r="M6" s="62">
         <f t="shared" si="7"/>
-        <v>0.006623988288</v>
+        <v>0.002820914396</v>
       </c>
       <c r="N6" s="62">
         <f t="shared" si="7"/>
-        <v>0.002820914396</v>
+        <v>0.003501418994</v>
       </c>
       <c r="O6" s="62">
         <f t="shared" si="7"/>
-        <v>0.003501418994</v>
+        <v>0.00249268835</v>
       </c>
       <c r="P6" s="62">
         <f t="shared" si="7"/>
-        <v>0.00249268835</v>
+        <v>0.009232208395</v>
       </c>
       <c r="Q6" s="62">
         <f t="shared" si="7"/>
-        <v>0.009232208395</v>
+        <v>0.001981574626</v>
       </c>
       <c r="R6" s="62">
         <f t="shared" si="7"/>
-        <v>0.001981574626</v>
+        <v>6902.440146</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B7" s="5" t="str">
         <f t="array" ref="B7">index($G$14:BO$14,0,MATCH(MIN(ABS(G7:R7)), ABS(G7:R7),0))</f>
@@ -33432,40 +33435,40 @@
       </c>
       <c r="K7" s="62">
         <f t="shared" si="8"/>
-        <v>0.002810350355</v>
+        <v>0.001400915928</v>
       </c>
       <c r="L7" s="62">
         <f t="shared" si="8"/>
-        <v>0.001400915928</v>
+        <v>0.00728422526</v>
       </c>
       <c r="M7" s="62">
         <f t="shared" si="8"/>
-        <v>0.00728422526</v>
+        <v>0</v>
       </c>
       <c r="N7" s="62">
         <f t="shared" si="8"/>
-        <v>0</v>
+        <v>0.0002512798999</v>
       </c>
       <c r="O7" s="62">
         <f t="shared" si="8"/>
-        <v>0.0002512798999</v>
+        <v>0.00008613811397</v>
       </c>
       <c r="P7" s="62">
         <f t="shared" si="8"/>
-        <v>0.00008613811397</v>
+        <v>0.006020419721</v>
       </c>
       <c r="Q7" s="62">
         <f t="shared" si="8"/>
-        <v>0.006020419721</v>
+        <v>0.0001421492138</v>
       </c>
       <c r="R7" s="62">
         <f t="shared" si="8"/>
-        <v>0.0001421492138</v>
+        <v>6911.096658</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B8" s="5" t="str">
         <f t="array" ref="B8">index($G$14:BO$14,0,MATCH(MIN(ABS(G8:R8)), ABS(G8:R8),0))</f>
@@ -33501,40 +33504,40 @@
       </c>
       <c r="K8" s="62">
         <f t="shared" si="9"/>
-        <v>0.001978149651</v>
+        <v>0.000650887213</v>
       </c>
       <c r="L8" s="62">
         <f t="shared" si="9"/>
-        <v>0.000650887213</v>
+        <v>0.008007623964</v>
       </c>
       <c r="M8" s="62">
         <f t="shared" si="9"/>
-        <v>0.008007623964</v>
+        <v>0.0001420418335</v>
       </c>
       <c r="N8" s="62">
         <f t="shared" si="9"/>
-        <v>0.0001420418335</v>
+        <v>0.0006989711991</v>
       </c>
       <c r="O8" s="62">
         <f t="shared" si="9"/>
-        <v>0.0006989711991</v>
+        <v>0.00002934267828</v>
       </c>
       <c r="P8" s="62">
         <f t="shared" si="9"/>
-        <v>0.00002934267828</v>
+        <v>0.007397906146</v>
       </c>
       <c r="Q8" s="62">
         <f t="shared" si="9"/>
-        <v>0.007397906146</v>
+        <v>0</v>
       </c>
       <c r="R8" s="62">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>6909.835266</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B9" s="5" t="str">
         <f t="array" ref="B9">index($G$14:BO$14,0,MATCH(MIN(ABS(G9:R9)), ABS(G9:R9),0))</f>
@@ -33570,40 +33573,40 @@
       </c>
       <c r="K9" s="62">
         <f t="shared" si="10"/>
-        <v>0.000655366939</v>
+        <v>0.00006158206588</v>
       </c>
       <c r="L9" s="62">
         <f t="shared" si="10"/>
-        <v>0.00006158206588</v>
+        <v>0.009043130794</v>
       </c>
       <c r="M9" s="62">
         <f t="shared" si="10"/>
-        <v>0.009043130794</v>
+        <v>0.001391576807</v>
       </c>
       <c r="N9" s="62">
         <f t="shared" si="10"/>
-        <v>0.001391576807</v>
+        <v>0.002413606947</v>
       </c>
       <c r="O9" s="62">
         <f t="shared" si="10"/>
-        <v>0.002413606947</v>
+        <v>0.0009417635615</v>
       </c>
       <c r="P9" s="62">
         <f t="shared" si="10"/>
-        <v>0.0009417635615</v>
+        <v>0.01018378288</v>
       </c>
       <c r="Q9" s="62">
         <f t="shared" si="10"/>
-        <v>0.01018378288</v>
+        <v>0.0006681975512</v>
       </c>
       <c r="R9" s="62">
         <f t="shared" si="10"/>
-        <v>0.0006681975512</v>
+        <v>6906.156012</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B10" s="5" t="str">
         <f t="array" ref="B10">index($G$14:BO$14,0,MATCH(MIN(ABS(G10:R10)), ABS(G10:R10),0))</f>
@@ -33639,40 +33642,40 @@
       </c>
       <c r="K10" s="62">
         <f t="shared" si="11"/>
-        <v>0.00109813081</v>
+        <v>0</v>
       </c>
       <c r="L10" s="62">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>0.01037753939</v>
       </c>
       <c r="M10" s="62">
         <f t="shared" si="11"/>
-        <v>0.01037753939</v>
+        <v>0.001400759249</v>
       </c>
       <c r="N10" s="62">
         <f t="shared" si="11"/>
-        <v>0.001400759249</v>
+        <v>0.002596410728</v>
       </c>
       <c r="O10" s="62">
         <f t="shared" si="11"/>
-        <v>0.002596410728</v>
+        <v>0.0008692858686</v>
       </c>
       <c r="P10" s="62">
         <f t="shared" si="11"/>
-        <v>0.0008692858686</v>
+        <v>0.01120593295</v>
       </c>
       <c r="Q10" s="62">
         <f t="shared" si="11"/>
-        <v>0.01120593295</v>
+        <v>0.0006507879887</v>
       </c>
       <c r="R10" s="62">
         <f t="shared" si="11"/>
-        <v>0.0006507879887</v>
+        <v>6907.034108</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B11" s="5" t="str">
         <f t="array" ref="B11">index($G$14:BO$14,0,MATCH(MIN(ABS(G11:R11)), ABS(G11:R11),0))</f>
@@ -33708,40 +33711,40 @@
       </c>
       <c r="K11" s="62">
         <f t="shared" si="12"/>
-        <v>0.002488806477</v>
+        <v>0.0008693372576</v>
       </c>
       <c r="L11" s="62">
         <f t="shared" si="12"/>
-        <v>0.0008693372576</v>
+        <v>0.008440878854</v>
       </c>
       <c r="M11" s="62">
         <f t="shared" si="12"/>
-        <v>0.008440878854</v>
+        <v>0.00008592434518</v>
       </c>
       <c r="N11" s="62">
         <f t="shared" si="12"/>
-        <v>0.00008592434518</v>
+        <v>0.0006268241261</v>
       </c>
       <c r="O11" s="62">
         <f t="shared" si="12"/>
-        <v>0.0006268241261</v>
+        <v>0</v>
       </c>
       <c r="P11" s="62">
         <f t="shared" si="12"/>
-        <v>0</v>
+        <v>0.007439583857</v>
       </c>
       <c r="Q11" s="62">
         <f t="shared" si="12"/>
-        <v>0.007439583857</v>
+        <v>0.00002923768412</v>
       </c>
       <c r="R11" s="62">
         <f t="shared" si="12"/>
-        <v>0.00002923768412</v>
+        <v>6910.734559</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B12" s="5" t="str">
         <f t="array" ref="B12">index($G$14:BO$14,0,MATCH(MIN(ABS(G12:R12)), ABS(G12:R12),0))</f>
@@ -33777,40 +33780,40 @@
       </c>
       <c r="K12" s="62">
         <f t="shared" si="13"/>
-        <v>0.00004811135125</v>
+        <v>0.0008033484</v>
       </c>
       <c r="L12" s="62">
         <f t="shared" si="13"/>
-        <v>0.0008033484</v>
+        <v>0.006389965451</v>
       </c>
       <c r="M12" s="62">
         <f t="shared" si="13"/>
-        <v>0.006389965451</v>
+        <v>0.002124188828</v>
       </c>
       <c r="N12" s="62">
         <f t="shared" si="13"/>
-        <v>0.002124188828</v>
+        <v>0.002748385528</v>
       </c>
       <c r="O12" s="62">
         <f t="shared" si="13"/>
-        <v>0.002748385528</v>
+        <v>0.001850510714</v>
       </c>
       <c r="P12" s="62">
         <f t="shared" si="13"/>
-        <v>0.001850510714</v>
+        <v>0.00848609105</v>
       </c>
       <c r="Q12" s="62">
         <f t="shared" si="13"/>
-        <v>0.00848609105</v>
+        <v>0.001414422628</v>
       </c>
       <c r="R12" s="62">
         <f t="shared" si="13"/>
-        <v>0.001414422628</v>
+        <v>6903.585085</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B13" s="5" t="str">
         <f t="array" ref="B13">index($G$14:BO$14,0,MATCH(MIN(ABS(G13:R13)), ABS(G13:R13),0))</f>
@@ -33846,35 +33849,35 @@
       </c>
       <c r="K13" s="62">
         <f t="shared" si="14"/>
-        <v>0.003479283563</v>
+        <v>0.002596766859</v>
       </c>
       <c r="L13" s="62">
         <f t="shared" si="14"/>
-        <v>0.002596766859</v>
+        <v>0.005383586454</v>
       </c>
       <c r="M13" s="62">
         <f t="shared" si="14"/>
-        <v>0.005383586454</v>
+        <v>0.0002517095076</v>
       </c>
       <c r="N13" s="62">
         <f t="shared" si="14"/>
-        <v>0.0002517095076</v>
+        <v>0</v>
       </c>
       <c r="O13" s="62">
         <f t="shared" si="14"/>
-        <v>0</v>
+        <v>0.0006274651317</v>
       </c>
       <c r="P13" s="62">
         <f t="shared" si="14"/>
-        <v>0.0006274651317</v>
+        <v>0.003865092331</v>
       </c>
       <c r="Q13" s="62">
         <f t="shared" si="14"/>
-        <v>0.003865092331</v>
+        <v>0.0006995026535</v>
       </c>
       <c r="R13" s="62">
         <f t="shared" si="14"/>
-        <v>0.0006995026535</v>
+        <v>6911.256665</v>
       </c>
     </row>
     <row r="14">
@@ -33883,7 +33886,7 @@
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
       <c r="F14" s="3" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="G14" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("transpose(filter(Monuments!A$2:A918,Monuments!B2:B918=""Corner""))"),"Acton/Boxborough/Littleton")</f>
@@ -33902,34 +33905,30 @@
         <v>Acton/Carlisle 2</v>
       </c>
       <c r="K14" s="5" t="str">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Acton/Carlisle/Concord")</f>
-        <v>Acton/Carlisle/Concord</v>
-      </c>
-      <c r="L14" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Acton/Carlisle/Westford")</f>
         <v>Acton/Carlisle/Westford</v>
       </c>
-      <c r="M14" s="5" t="str">
+      <c r="L14" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Acton/Concord/Maynard/Sudbury")</f>
         <v>Acton/Concord/Maynard/Sudbury</v>
       </c>
-      <c r="N14" s="5" t="str">
+      <c r="M14" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Acton/Littleton 1")</f>
         <v>Acton/Littleton 1</v>
       </c>
-      <c r="O14" s="5" t="str">
+      <c r="N14" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Acton/Littleton 2")</f>
         <v>Acton/Littleton 2</v>
       </c>
-      <c r="P14" s="5" t="str">
+      <c r="O14" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Acton/Littleton/Westford")</f>
         <v>Acton/Littleton/Westford</v>
       </c>
-      <c r="Q14" s="5" t="str">
+      <c r="P14" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Acton/Maynard/Stow")</f>
         <v>Acton/Maynard/Stow</v>
       </c>
-      <c r="R14" s="5" t="str">
+      <c r="Q14" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"Acton/Westford")</f>
         <v>Acton/Westford</v>
       </c>
@@ -33940,7 +33939,7 @@
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
       <c r="F15" s="3" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="G15" s="3">
         <f>IFERROR(__xludf.DUMMYFUNCTION("transpose(filter(Monuments!X$2:X918,Monuments!B2:B918=""Corner""))"),-71.473529496)</f>
@@ -33959,34 +33958,30 @@
         <v>-71.39794715</v>
       </c>
       <c r="K15" s="5">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-71.385158)</f>
-        <v>-71.385158</v>
-      </c>
-      <c r="L15" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-71.399515336)</f>
         <v>-71.39951534</v>
       </c>
-      <c r="M15" s="5">
+      <c r="L15" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-71.430394779)</f>
         <v>-71.43039478</v>
       </c>
-      <c r="N15" s="5">
+      <c r="M15" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-71.435017906)</f>
         <v>-71.43501791</v>
       </c>
-      <c r="O15" s="5">
+      <c r="N15" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-71.443940303)</f>
         <v>-71.4439403</v>
       </c>
-      <c r="P15" s="5">
+      <c r="O15" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-71.428534514)</f>
         <v>-71.42853451</v>
       </c>
-      <c r="Q15" s="5">
+      <c r="P15" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-71.4643289959999)</f>
         <v>-71.464329</v>
       </c>
-      <c r="R15" s="5">
+      <c r="Q15" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),-71.42379555)</f>
         <v>-71.42379555</v>
       </c>
@@ -33997,7 +33992,7 @@
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
       <c r="F16" s="3" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="G16" s="63">
         <f>IFERROR(__xludf.DUMMYFUNCTION("transpose(filter(Monuments!T$2:T918,Monuments!B2:B918=""Corner""))"),42.5001860150001)</f>
@@ -34016,41 +34011,37 @@
         <v>42.52634481</v>
       </c>
       <c r="K16" s="5">
-        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),42.504159)</f>
-        <v>42.504159</v>
-      </c>
-      <c r="L16" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),42.534025086)</f>
         <v>42.53402509</v>
       </c>
-      <c r="M16" s="5">
+      <c r="L16" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),42.436947994)</f>
         <v>42.43694799</v>
       </c>
-      <c r="N16" s="5">
+      <c r="M16" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),42.5221791480001)</f>
         <v>42.52217915</v>
       </c>
-      <c r="O16" s="5">
+      <c r="N16" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),42.509068563)</f>
         <v>42.50906856</v>
       </c>
-      <c r="P16" s="5">
+      <c r="O16" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),42.528812154)</f>
         <v>42.52881215</v>
       </c>
-      <c r="Q16" s="5">
+      <c r="P16" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),42.4503286410001)</f>
         <v>42.45032864</v>
       </c>
-      <c r="R16" s="5">
+      <c r="Q16" s="5">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),42.5261982760001)</f>
         <v>42.52619828</v>
       </c>
     </row>
     <row r="17">
       <c r="F17" s="3" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="G17" s="5" t="str">
         <f t="shared" ref="G17:R17" si="15">vlookup(G$14,$B:$E,4,False)</f>
@@ -34062,7 +34053,7 @@
       </c>
       <c r="I17" s="5" t="str">
         <f t="shared" si="15"/>
-        <v>-71.3915635</v>
+        <v>-71.3849469</v>
       </c>
       <c r="J17" s="5" t="str">
         <f t="shared" si="15"/>
@@ -34070,40 +34061,40 @@
       </c>
       <c r="K17" s="5" t="str">
         <f t="shared" si="15"/>
-        <v>-71.3849469</v>
+        <v>-71.3995154</v>
       </c>
       <c r="L17" s="5" t="str">
         <f t="shared" si="15"/>
-        <v>-71.3995154</v>
+        <v>-71.4303980</v>
       </c>
       <c r="M17" s="5" t="str">
         <f t="shared" si="15"/>
-        <v>-71.4303980</v>
+        <v>-71.4350172</v>
       </c>
       <c r="N17" s="5" t="str">
         <f t="shared" si="15"/>
-        <v>-71.4350172</v>
+        <v>-71.4439395</v>
       </c>
       <c r="O17" s="5" t="str">
         <f t="shared" si="15"/>
-        <v>-71.4439395</v>
+        <v>-71.4285338</v>
       </c>
       <c r="P17" s="5" t="str">
         <f t="shared" si="15"/>
-        <v>-71.4285338</v>
+        <v>-71.4643296</v>
       </c>
       <c r="Q17" s="5" t="str">
         <f t="shared" si="15"/>
-        <v>-71.4643296</v>
+        <v>-71.4237948</v>
       </c>
       <c r="R17" s="5" t="str">
         <f t="shared" si="15"/>
-        <v>-71.4237948</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="18">
       <c r="F18" s="3" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="G18" s="5" t="str">
         <f t="shared" ref="G18:R18" si="16">vlookup(G$14,$B:$E,3,False)</f>
@@ -34115,7 +34106,7 @@
       </c>
       <c r="I18" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>42.5068200</v>
+        <v>42.5044645</v>
       </c>
       <c r="J18" s="5" t="str">
         <f t="shared" si="16"/>
@@ -34123,40 +34114,40 @@
       </c>
       <c r="K18" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>42.5044645</v>
+        <v>42.5340253</v>
       </c>
       <c r="L18" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>42.5340253</v>
+        <v>42.4369486</v>
       </c>
       <c r="M18" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>42.4369486</v>
+        <v>42.5221704</v>
       </c>
       <c r="N18" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>42.5221704</v>
+        <v>42.5090599</v>
       </c>
       <c r="O18" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>42.5090599</v>
+        <v>42.5288034</v>
       </c>
       <c r="P18" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>42.5288034</v>
+        <v>42.4503310</v>
       </c>
       <c r="Q18" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>42.4503310</v>
+        <v>42.5261896</v>
       </c>
       <c r="R18" s="5" t="str">
         <f t="shared" si="16"/>
-        <v>42.5261896</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="19">
       <c r="F19" s="3" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="G19" s="64">
         <f t="shared" ref="G19:R19" si="17">G17-G15</f>
@@ -34168,7 +34159,7 @@
       </c>
       <c r="I19" s="64">
         <f t="shared" si="17"/>
-        <v>0.0000006859999928</v>
+        <v>0.006617286</v>
       </c>
       <c r="J19" s="64">
         <f t="shared" si="17"/>
@@ -34176,40 +34167,40 @@
       </c>
       <c r="K19" s="64">
         <f t="shared" si="17"/>
-        <v>0.0002111</v>
+        <v>-0.0000000640000053</v>
       </c>
       <c r="L19" s="64">
         <f t="shared" si="17"/>
-        <v>-0.0000000640000053</v>
+        <v>-0.000003221</v>
       </c>
       <c r="M19" s="64">
         <f t="shared" si="17"/>
-        <v>-0.000003221</v>
+        <v>0.0000007059999945</v>
       </c>
       <c r="N19" s="64">
         <f t="shared" si="17"/>
-        <v>0.0000007059999945</v>
+        <v>0.000000803000006</v>
       </c>
       <c r="O19" s="64">
         <f t="shared" si="17"/>
-        <v>0.000000803000006</v>
+        <v>0.0000007140000093</v>
       </c>
       <c r="P19" s="64">
         <f t="shared" si="17"/>
-        <v>0.0000007140000093</v>
+        <v>-0.0000006040000926</v>
       </c>
       <c r="Q19" s="64">
         <f t="shared" si="17"/>
-        <v>-0.0000006040000926</v>
-      </c>
-      <c r="R19" s="64">
+        <v>0.0000007499999981</v>
+      </c>
+      <c r="R19" s="64" t="str">
         <f t="shared" si="17"/>
-        <v>0.0000007499999981</v>
+        <v>#N/A</v>
       </c>
     </row>
     <row r="20">
       <c r="F20" s="3" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="G20" s="64">
         <f t="shared" ref="G20:R20" si="18">G18-G16</f>
@@ -34221,7 +34212,7 @@
       </c>
       <c r="I20" s="64">
         <f t="shared" si="18"/>
-        <v>-0.000008708000102</v>
+        <v>-0.002364208</v>
       </c>
       <c r="J20" s="64">
         <f t="shared" si="18"/>
@@ -34229,35 +34220,35 @@
       </c>
       <c r="K20" s="64">
         <f t="shared" si="18"/>
-        <v>0.0003055</v>
+        <v>0.0000002140000035</v>
       </c>
       <c r="L20" s="64">
         <f t="shared" si="18"/>
-        <v>0.0000002140000035</v>
+        <v>0.0000006060000004</v>
       </c>
       <c r="M20" s="64">
         <f t="shared" si="18"/>
-        <v>0.0000006060000004</v>
+        <v>-0.000008748000099</v>
       </c>
       <c r="N20" s="64">
         <f t="shared" si="18"/>
-        <v>-0.000008748000099</v>
+        <v>-0.000008663000003</v>
       </c>
       <c r="O20" s="64">
         <f t="shared" si="18"/>
-        <v>-0.000008663000003</v>
+        <v>-0.000008754</v>
       </c>
       <c r="P20" s="64">
         <f t="shared" si="18"/>
-        <v>-0.000008754</v>
+        <v>0.0000023589999</v>
       </c>
       <c r="Q20" s="64">
         <f t="shared" si="18"/>
-        <v>0.0000023589999</v>
-      </c>
-      <c r="R20" s="64">
+        <v>-0.0000086760001</v>
+      </c>
+      <c r="R20" s="64" t="str">
         <f t="shared" si="18"/>
-        <v>-0.0000086760001</v>
+        <v>#N/A</v>
       </c>
     </row>
   </sheetData>
@@ -34290,7 +34281,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="B2" s="22">
         <v>42.5001860150001</v>
@@ -34301,7 +34292,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B3" s="22">
         <v>42.4637837510001</v>
@@ -34312,7 +34303,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B4" s="22">
         <v>42.5068287080001</v>
@@ -34323,7 +34314,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B5" s="22">
         <v>42.526344807</v>
@@ -34334,7 +34325,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B6" s="22">
         <v>42.504473137</v>
@@ -34345,7 +34336,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B7" s="22">
         <v>42.534025086</v>
@@ -34356,7 +34347,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B8" s="22">
         <v>42.436947994</v>
@@ -34367,7 +34358,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B9" s="22">
         <v>42.5221791480001</v>
@@ -34378,7 +34369,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B10" s="22">
         <v>42.509068563</v>
@@ -34389,7 +34380,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B11" s="22">
         <v>42.528812154</v>
@@ -34400,7 +34391,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B12" s="22">
         <v>42.4503286410001</v>
@@ -34411,7 +34402,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B13" s="22">
         <v>42.5261982760001</v>

</xml_diff>

<commit_message>
Acton Bounds.xlsx: add Fort Pond Road westerly-monument note (Order 30)
Notes on location for the Acton/Littleton Fort Pond Road crossing: what
was found is most likely the westerly of the two monuments the 1904 survey
describes on the Cash Road; the easterly one would sit closer to the true
boundary line, explaining the ~8.6m distance-to-line offset. Only real cell
change vs HEAD (Monuments!P29); For Mapping!Q28 is its cached-value copy.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Acton Bounds.xlsx
+++ b/Acton Bounds.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="926" uniqueCount="537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="927" uniqueCount="538">
   <si>
     <t>Count by status/town</t>
   </si>
@@ -625,6 +625,9 @@
   </si>
   <si>
     <t>Fort Pond Road</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What we found is most likely the westerly of two monuments. The easterly monument would have been much closer to the actual boundary line. </t>
   </si>
   <si>
     <t>The easterly and westerly sides of the Cash road</t>
@@ -4748,16 +4751,18 @@
       <c r="O29" s="15">
         <v>45810.0</v>
       </c>
-      <c r="P29" s="1"/>
+      <c r="P29" s="1" t="s">
+        <v>201</v>
+      </c>
       <c r="Q29" s="16" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="R29" s="1"/>
       <c r="S29" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T29" s="24" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="U29" s="5">
         <f t="shared" si="36"/>
@@ -4772,7 +4777,7 @@
         <v>21.5496</v>
       </c>
       <c r="X29" s="24" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="Y29" s="5">
         <f t="shared" si="39"/>
@@ -4819,7 +4824,7 @@
         <v>45810.0</v>
       </c>
       <c r="P30" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="Q30" s="1" t="s">
         <v>74</v>
@@ -4829,7 +4834,7 @@
         <v>69</v>
       </c>
       <c r="T30" s="17" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="U30" s="5">
         <f t="shared" si="36"/>
@@ -4844,7 +4849,7 @@
         <v>21.072</v>
       </c>
       <c r="X30" s="17" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="Y30" s="5">
         <f>abs(trunc(X30))</f>
@@ -4878,10 +4883,10 @@
         <v>53</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="L31" s="1" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="M31" s="4"/>
       <c r="N31" s="1" t="s">
@@ -4891,7 +4896,7 @@
         <v>45741.0</v>
       </c>
       <c r="P31" s="1" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Q31" s="1" t="s">
         <v>74</v>
@@ -4901,7 +4906,7 @@
         <v>69</v>
       </c>
       <c r="T31" s="17" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="U31" s="5">
         <f>if(isblank(T31),"",abs(trunc(T31)))</f>
@@ -4916,7 +4921,7 @@
         <v>4.0788</v>
       </c>
       <c r="X31" s="17" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="Y31" s="5">
         <f>if(isblank(X31),"",abs(trunc(X31)))</f>
@@ -4966,16 +4971,16 @@
         <v>45810.0</v>
       </c>
       <c r="P32" s="1" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="Q32" s="16" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="S32" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T32" s="24" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="U32" s="5">
         <f t="shared" ref="U32:U37" si="42">abs(trunc(T32))</f>
@@ -4990,7 +4995,7 @@
         <v>26.7372</v>
       </c>
       <c r="X32" s="24" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="Y32" s="5">
         <f t="shared" ref="Y32:Y33" si="45">abs(trunc(X32))</f>
@@ -5037,7 +5042,7 @@
         <v>45810.0</v>
       </c>
       <c r="P33" s="1" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="Q33" s="1" t="s">
         <v>74</v>
@@ -5047,7 +5052,7 @@
         <v>69</v>
       </c>
       <c r="T33" s="17" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="U33" s="5">
         <f t="shared" si="42"/>
@@ -5062,7 +5067,7 @@
         <v>19.74</v>
       </c>
       <c r="X33" s="17" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="Y33" s="5">
         <f t="shared" si="45"/>
@@ -5099,10 +5104,10 @@
         <v>83</v>
       </c>
       <c r="L34" s="1" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="N34" s="1" t="s">
         <v>13</v>
@@ -5112,14 +5117,14 @@
       </c>
       <c r="P34" s="1"/>
       <c r="Q34" s="16" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="R34" s="4"/>
       <c r="S34" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T34" s="17" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="U34" s="5">
         <f t="shared" si="42"/>
@@ -5134,7 +5139,7 @@
         <v>5.1012</v>
       </c>
       <c r="X34" s="17" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="Y34" s="5">
         <f t="shared" ref="Y34:Y36" si="48">if(isblank(X34),"",abs(trunc(X34)))</f>
@@ -5168,7 +5173,7 @@
         <v>53</v>
       </c>
       <c r="K35" s="1" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="L35" s="1"/>
       <c r="M35" s="4"/>
@@ -5179,7 +5184,7 @@
         <v>45810.0</v>
       </c>
       <c r="P35" s="1" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="Q35" s="1" t="s">
         <v>74</v>
@@ -5189,7 +5194,7 @@
         <v>69</v>
       </c>
       <c r="T35" s="17" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="U35" s="5">
         <f t="shared" si="42"/>
@@ -5204,7 +5209,7 @@
         <v>18.972</v>
       </c>
       <c r="X35" s="17" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="Y35" s="5">
         <f t="shared" si="48"/>
@@ -5226,7 +5231,7 @@
         <v>32.0</v>
       </c>
       <c r="AE35" s="3" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="36">
@@ -5241,7 +5246,7 @@
         <v>53</v>
       </c>
       <c r="K36" s="1" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="L36" s="1" t="s">
         <v>200</v>
@@ -5254,19 +5259,19 @@
         <v>45810.0</v>
       </c>
       <c r="P36" s="1" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="Q36" s="16" t="s">
         <v>74</v>
       </c>
       <c r="R36" s="1" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="S36" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T36" s="24" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="U36" s="5">
         <f t="shared" si="42"/>
@@ -5281,7 +5286,7 @@
         <v>22.3236</v>
       </c>
       <c r="X36" s="24" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="Y36" s="5">
         <f t="shared" si="48"/>
@@ -5303,7 +5308,7 @@
         <v>31.0</v>
       </c>
       <c r="AE36" s="3" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
     </row>
     <row r="37">
@@ -5321,13 +5326,13 @@
         <v>53</v>
       </c>
       <c r="K37" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="L37" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="N37" s="1" t="s">
         <v>13</v>
@@ -5336,13 +5341,13 @@
         <v>45924.0</v>
       </c>
       <c r="P37" s="1" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="Q37" s="16" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="R37" s="1" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="S37" s="3" t="s">
         <v>87</v>
@@ -5397,30 +5402,30 @@
         <v>53</v>
       </c>
       <c r="K38" s="1" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="L38" s="1"/>
       <c r="M38" s="1" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N38" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O38" s="26" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P38" s="1" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="Q38" s="1" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="R38" s="1"/>
       <c r="S38" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T38" s="24" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="U38" s="5">
         <f t="shared" ref="U38:U41" si="51">if(isblank(T38),"",abs(trunc(T38)))</f>
@@ -5435,7 +5440,7 @@
         <v>44.5236</v>
       </c>
       <c r="X38" s="27" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="Y38" s="5">
         <f t="shared" ref="Y38:Y41" si="54">if(isblank(X38),"",abs(trunc(X38)))</f>
@@ -5472,29 +5477,29 @@
         <v>103</v>
       </c>
       <c r="L39" s="1" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="N39" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O39" s="26" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P39" s="1" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="Q39" s="1" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="R39" s="1"/>
       <c r="S39" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T39" s="28" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="U39" s="5">
         <f t="shared" si="51"/>
@@ -5509,7 +5514,7 @@
         <v>46.428</v>
       </c>
       <c r="X39" s="27" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="Y39" s="5">
         <f t="shared" si="54"/>
@@ -5531,7 +5536,7 @@
         <v>47.0</v>
       </c>
       <c r="AE39" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
     </row>
     <row r="40">
@@ -5546,34 +5551,34 @@
         <v>53</v>
       </c>
       <c r="K40" s="1" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L40" s="1" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="N40" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O40" s="26" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P40" s="1" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="Q40" s="1" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="R40" s="1" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="S40" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T40" s="17" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="U40" s="5">
         <f t="shared" si="51"/>
@@ -5588,7 +5593,7 @@
         <v>32.2044</v>
       </c>
       <c r="X40" s="27" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="Y40" s="5">
         <f t="shared" si="54"/>
@@ -5610,7 +5615,7 @@
         <v>49.0</v>
       </c>
       <c r="AE40" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
     </row>
     <row r="41">
@@ -5629,7 +5634,7 @@
       </c>
       <c r="L41" s="1"/>
       <c r="M41" s="1" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="N41" s="1" t="s">
         <v>12</v>
@@ -5638,17 +5643,17 @@
         <v>45770.0</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="Q41" s="1" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="R41" s="4"/>
       <c r="S41" s="3" t="s">
         <v>69</v>
       </c>
       <c r="T41" s="17" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="U41" s="5">
         <f t="shared" si="51"/>
@@ -5663,7 +5668,7 @@
         <v>20.076</v>
       </c>
       <c r="X41" s="17" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="Y41" s="5">
         <f t="shared" si="54"/>
@@ -5685,7 +5690,7 @@
         <v>50.0</v>
       </c>
       <c r="AE41" s="3" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
     </row>
     <row r="42">
@@ -5700,13 +5705,13 @@
         <v>53</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="L42" s="1" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="N42" s="1" t="s">
         <v>12</v>
@@ -5715,17 +5720,17 @@
         <v>45862.0</v>
       </c>
       <c r="P42" s="1" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="Q42" s="1" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="R42" s="4"/>
       <c r="S42" s="3" t="s">
         <v>69</v>
       </c>
       <c r="T42" s="17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="U42" s="5">
         <f t="shared" ref="U42:U43" si="57">abs(trunc(T42))</f>
@@ -5740,7 +5745,7 @@
         <v>13.7328</v>
       </c>
       <c r="X42" s="17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="Y42" s="5">
         <f t="shared" ref="Y42:Y50" si="60">abs(trunc(X42))</f>
@@ -5762,7 +5767,7 @@
         <v>51.0</v>
       </c>
       <c r="AE42" s="3" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
     </row>
     <row r="43">
@@ -5780,23 +5785,23 @@
         <v>53</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="L43" s="1"/>
       <c r="M43" s="1" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="N43" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O43" s="26" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="P43" s="1" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="Q43" s="1" t="s">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="R43" s="1"/>
       <c r="S43" s="3" t="s">
@@ -5852,7 +5857,7 @@
         <v>53</v>
       </c>
       <c r="K44" s="1" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="L44" s="1"/>
       <c r="M44" s="4"/>
@@ -5860,20 +5865,20 @@
         <v>13</v>
       </c>
       <c r="O44" s="26" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P44" s="1" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="Q44" s="1" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="R44" s="1"/>
       <c r="S44" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T44" s="17" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="U44" s="5">
         <f t="shared" ref="U44:U46" si="63">if(isblank(T44),"",abs(trunc(T44)))</f>
@@ -5888,7 +5893,7 @@
         <v>5.4108</v>
       </c>
       <c r="X44" s="17" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="Y44" s="5">
         <f t="shared" si="60"/>
@@ -5922,32 +5927,32 @@
         <v>53</v>
       </c>
       <c r="K45" s="1" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="L45" s="1" t="s">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="N45" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O45" s="26" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P45" s="1" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="Q45" s="1" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="R45" s="1"/>
       <c r="S45" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T45" s="17" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="U45" s="5">
         <f t="shared" si="63"/>
@@ -5962,7 +5967,7 @@
         <v>12.204</v>
       </c>
       <c r="X45" s="17" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="Y45" s="5">
         <f t="shared" si="60"/>
@@ -5996,30 +6001,30 @@
         <v>53</v>
       </c>
       <c r="K46" s="1" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="L46" s="1" t="s">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="M46" s="4"/>
       <c r="N46" s="1" t="s">
         <v>13</v>
       </c>
       <c r="O46" s="26" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P46" s="1" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="Q46" s="1" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="R46" s="1"/>
       <c r="S46" s="3" t="s">
         <v>57</v>
       </c>
       <c r="T46" s="17" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="U46" s="5">
         <f t="shared" si="63"/>
@@ -6034,7 +6039,7 @@
         <v>34.8912</v>
       </c>
       <c r="X46" s="17" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="Y46" s="5">
         <f t="shared" si="60"/>
@@ -6068,11 +6073,11 @@
         <v>53</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L47" s="1"/>
       <c r="M47" s="1" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="N47" s="1" t="s">
         <v>12</v>
@@ -6081,10 +6086,10 @@
         <v>45580.0</v>
       </c>
       <c r="P47" s="1" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="Q47" s="1" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="R47" s="1"/>
       <c r="S47" s="3" t="s">
@@ -6128,7 +6133,7 @@
         <v>20.0</v>
       </c>
       <c r="AE47" s="3" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
     </row>
     <row r="48">
@@ -6143,7 +6148,7 @@
         <v>53</v>
       </c>
       <c r="K48" s="1" t="s">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="L48" s="1"/>
       <c r="M48" s="4"/>
@@ -6154,7 +6159,7 @@
         <v>45580.0</v>
       </c>
       <c r="P48" s="1" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="Q48" s="1" t="s">
         <v>74</v>
@@ -6164,7 +6169,7 @@
         <v>69</v>
       </c>
       <c r="T48" s="17" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="U48" s="5">
         <f t="shared" si="66"/>
@@ -6179,7 +6184,7 @@
         <v>34.5144</v>
       </c>
       <c r="X48" s="17" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="Y48" s="5">
         <f t="shared" si="60"/>
@@ -6216,7 +6221,7 @@
         <v>53</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="L49" s="1"/>
       <c r="M49" s="4"/>
@@ -6227,7 +6232,7 @@
         <v>45580.0</v>
       </c>
       <c r="P49" s="1" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="Q49" s="1" t="s">
         <v>74</v>
@@ -6237,7 +6242,7 @@
         <v>69</v>
       </c>
       <c r="T49" s="17" t="s">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="U49" s="5">
         <f t="shared" si="66"/>
@@ -6252,7 +6257,7 @@
         <v>37.398</v>
       </c>
       <c r="X49" s="17" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="Y49" s="5">
         <f t="shared" si="60"/>
@@ -6286,7 +6291,7 @@
         <v>53</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="L50" s="1"/>
       <c r="M50" s="4"/>
@@ -6295,19 +6300,19 @@
       </c>
       <c r="O50" s="15"/>
       <c r="P50" s="1" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="Q50" s="1" t="s">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="R50" s="1" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="S50" s="3" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="T50" s="17" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="U50" s="5">
         <f t="shared" si="66"/>
@@ -6322,7 +6327,7 @@
         <v>51.042</v>
       </c>
       <c r="X50" s="17" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="Y50" s="5">
         <f t="shared" si="60"/>
@@ -6344,7 +6349,7 @@
         <v>18.0</v>
       </c>
       <c r="AE50" s="3" t="s">
-        <v>317</v>
+        <v>318</v>
       </c>
     </row>
     <row r="51">
@@ -6356,7 +6361,7 @@
         <v>52</v>
       </c>
       <c r="E51" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="K51" s="1" t="s">
         <v>111</v>
@@ -6368,10 +6373,10 @@
       </c>
       <c r="O51" s="15"/>
       <c r="P51" s="1" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="Q51" s="1" t="s">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="R51" s="4"/>
       <c r="T51" s="17"/>
@@ -6388,7 +6393,7 @@
         <v>23.0</v>
       </c>
       <c r="AE51" s="3" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
     </row>
     <row r="52">
@@ -6403,13 +6408,13 @@
         <v>53</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="L52" s="1" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="M52" s="1" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="N52" s="1" t="s">
         <v>12</v>
@@ -6418,17 +6423,17 @@
         <v>45580.0</v>
       </c>
       <c r="P52" s="1" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="Q52" s="1" t="s">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="R52" s="4"/>
       <c r="S52" s="3" t="s">
         <v>69</v>
       </c>
       <c r="T52" s="17" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="U52" s="5">
         <f>abs(trunc(T52))</f>
@@ -6443,7 +6448,7 @@
         <v>39.2664</v>
       </c>
       <c r="X52" s="17" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="Y52" s="5">
         <f>abs(trunc(X52))</f>
@@ -6465,7 +6470,7 @@
         <v>22.0</v>
       </c>
       <c r="AE52" s="3" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
     </row>
     <row r="53">
@@ -21536,10 +21541,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="32" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="B1" s="32" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="C1" s="33"/>
       <c r="D1" s="33"/>
@@ -21759,230 +21764,230 @@
     </row>
     <row r="12" ht="22.5" customHeight="1">
       <c r="A12" s="39" t="s">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="B12" s="39" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C12" s="39" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="D12" s="39" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="E12" s="40" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="F12" s="40" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="G12" s="40" t="s">
         <v>180</v>
       </c>
       <c r="H12" s="40" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="I12" s="40" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="J12" s="40" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="K12" s="40" t="s">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="L12" s="40" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="M12" s="10"/>
     </row>
     <row r="13" ht="22.5" customHeight="1">
       <c r="A13" s="41" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="B13" s="41" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C13" s="41" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D13" s="42"/>
       <c r="E13" s="41" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F13" s="43" t="s">
+        <v>343</v>
+      </c>
+      <c r="G13" s="43" t="s">
+        <v>343</v>
+      </c>
+      <c r="H13" s="43" t="s">
+        <v>343</v>
+      </c>
+      <c r="I13" s="43" t="s">
+        <v>343</v>
+      </c>
+      <c r="J13" s="43" t="s">
+        <v>343</v>
+      </c>
+      <c r="K13" s="43" t="s">
+        <v>343</v>
+      </c>
+      <c r="L13" s="43" t="s">
         <v>342</v>
-      </c>
-      <c r="G13" s="43" t="s">
-        <v>342</v>
-      </c>
-      <c r="H13" s="43" t="s">
-        <v>342</v>
-      </c>
-      <c r="I13" s="43" t="s">
-        <v>342</v>
-      </c>
-      <c r="J13" s="43" t="s">
-        <v>342</v>
-      </c>
-      <c r="K13" s="43" t="s">
-        <v>342</v>
-      </c>
-      <c r="L13" s="43" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="14" ht="22.5" customHeight="1">
       <c r="A14" s="44" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="B14" s="44" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="C14" s="44" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="D14" s="45"/>
       <c r="E14" s="44" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F14" s="46" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="G14" s="46" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="H14" s="46" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="I14" s="46" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="J14" s="46" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K14" s="46" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="L14" s="45"/>
     </row>
     <row r="15" ht="22.5" customHeight="1">
       <c r="A15" s="41" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="B15" s="41" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="C15" s="41" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="D15" s="42"/>
       <c r="E15" s="41" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F15" s="47" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="G15" s="47" t="s">
+        <v>350</v>
+      </c>
+      <c r="H15" s="47" t="s">
+        <v>350</v>
+      </c>
+      <c r="I15" s="47" t="s">
+        <v>350</v>
+      </c>
+      <c r="J15" s="47" t="s">
         <v>349</v>
       </c>
-      <c r="H15" s="47" t="s">
-        <v>349</v>
-      </c>
-      <c r="I15" s="47" t="s">
-        <v>349</v>
-      </c>
-      <c r="J15" s="47" t="s">
-        <v>348</v>
-      </c>
       <c r="K15" s="47" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="L15" s="42"/>
     </row>
     <row r="16" ht="22.5" customHeight="1">
       <c r="A16" s="44" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="B16" s="44" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C16" s="44" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D16" s="45"/>
       <c r="E16" s="44" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F16" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="G16" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H16" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="I16" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J16" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K16" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="L16" s="45"/>
     </row>
     <row r="17" ht="22.5" customHeight="1">
       <c r="A17" s="41" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="B17" s="41" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="C17" s="41" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="D17" s="42"/>
       <c r="E17" s="41" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F17" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G17" s="47" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H17" s="47" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="I17" s="47" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J17" s="47" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K17" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="L17" s="42"/>
     </row>
     <row r="18" ht="22.5" customHeight="1">
       <c r="A18" s="44" t="s">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B18" s="44" t="s">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C18" s="44" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D18" s="44" t="s">
         <v>2</v>
       </c>
       <c r="E18" s="44" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F18" s="45"/>
       <c r="G18" s="45"/>
@@ -21990,25 +21995,25 @@
       <c r="I18" s="45"/>
       <c r="J18" s="45"/>
       <c r="K18" s="46" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="L18" s="45"/>
     </row>
     <row r="19" ht="22.5" customHeight="1">
       <c r="A19" s="41" t="s">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="B19" s="41" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="C19" s="41" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="D19" s="41" t="s">
         <v>2</v>
       </c>
       <c r="E19" s="41" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F19" s="42"/>
       <c r="G19" s="42"/>
@@ -22016,25 +22021,25 @@
       <c r="I19" s="42"/>
       <c r="J19" s="42"/>
       <c r="K19" s="47" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="L19" s="42"/>
     </row>
     <row r="20" ht="22.5" customHeight="1">
       <c r="A20" s="44" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="B20" s="44" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C20" s="44" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="D20" s="44" t="s">
         <v>2</v>
       </c>
       <c r="E20" s="44" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="F20" s="45"/>
       <c r="G20" s="45"/>
@@ -22042,65 +22047,65 @@
       <c r="I20" s="45"/>
       <c r="J20" s="45"/>
       <c r="K20" s="46" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L20" s="45"/>
     </row>
     <row r="21" ht="22.5" customHeight="1">
       <c r="A21" s="41" t="s">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="B21" s="41" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C21" s="41" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="D21" s="42"/>
       <c r="E21" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="F21" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="G21" s="47" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="H21" s="47" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="I21" s="48" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="J21" s="48" t="s">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="K21" s="48" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="L21" s="42"/>
     </row>
     <row r="22" ht="22.5" customHeight="1">
       <c r="A22" s="46" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="B22" s="46" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="C22" s="45"/>
       <c r="D22" s="46" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E22" s="45"/>
       <c r="F22" s="45"/>
       <c r="G22" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H22" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="I22" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J22" s="45"/>
       <c r="K22" s="45"/>
@@ -22108,25 +22113,25 @@
     </row>
     <row r="23" ht="22.5" customHeight="1">
       <c r="A23" s="47" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="B23" s="47" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="C23" s="42"/>
       <c r="D23" s="47" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E23" s="42"/>
       <c r="F23" s="42"/>
       <c r="G23" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="H23" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="I23" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J23" s="42"/>
       <c r="K23" s="42"/>
@@ -22134,25 +22139,25 @@
     </row>
     <row r="24" ht="22.5" customHeight="1">
       <c r="A24" s="46" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="B24" s="46" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="C24" s="45"/>
       <c r="D24" s="46" t="s">
-        <v>372</v>
+        <v>373</v>
       </c>
       <c r="E24" s="45"/>
       <c r="F24" s="45"/>
       <c r="G24" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H24" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="I24" s="49" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J24" s="50"/>
       <c r="K24" s="50"/>
@@ -22160,10 +22165,10 @@
     </row>
     <row r="25" ht="22.5" customHeight="1">
       <c r="A25" s="47" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="B25" s="47" t="s">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="C25" s="42"/>
       <c r="D25" s="47" t="s">
@@ -22172,13 +22177,13 @@
       <c r="E25" s="42"/>
       <c r="F25" s="42"/>
       <c r="G25" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="H25" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="I25" s="48" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J25" s="51"/>
       <c r="K25" s="51"/>
@@ -22186,13 +22191,13 @@
     </row>
     <row r="26" ht="22.5" customHeight="1">
       <c r="A26" s="46" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="B26" s="46" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="C26" s="45" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="D26" s="46" t="s">
         <v>6</v>
@@ -22200,11 +22205,11 @@
       <c r="E26" s="50"/>
       <c r="F26" s="45"/>
       <c r="G26" s="46" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="H26" s="45"/>
       <c r="I26" s="49" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J26" s="45"/>
       <c r="K26" s="45"/>
@@ -22212,13 +22217,13 @@
     </row>
     <row r="27" ht="22.5" customHeight="1">
       <c r="A27" s="47" t="s">
-        <v>382</v>
+        <v>383</v>
       </c>
       <c r="B27" s="47" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="C27" s="42" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="D27" s="47" t="s">
         <v>6</v>
@@ -22226,11 +22231,11 @@
       <c r="E27" s="51"/>
       <c r="F27" s="42"/>
       <c r="G27" s="47" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="H27" s="42"/>
       <c r="I27" s="48" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="J27" s="42"/>
       <c r="K27" s="42"/>
@@ -22238,10 +22243,10 @@
     </row>
     <row r="28" ht="22.5" customHeight="1">
       <c r="A28" s="46" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="B28" s="46" t="s">
-        <v>386</v>
+        <v>387</v>
       </c>
       <c r="C28" s="45"/>
       <c r="D28" s="46" t="s">
@@ -22250,26 +22255,26 @@
       <c r="E28" s="45"/>
       <c r="F28" s="45"/>
       <c r="G28" s="46" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="H28" s="46" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="I28" s="46" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J28" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K28" s="45"/>
       <c r="L28" s="45"/>
     </row>
     <row r="29" ht="22.5" customHeight="1">
       <c r="A29" s="47" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="B29" s="47" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="C29" s="42"/>
       <c r="D29" s="47" t="s">
@@ -22278,26 +22283,26 @@
       <c r="E29" s="42"/>
       <c r="F29" s="42"/>
       <c r="G29" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="H29" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="I29" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J29" s="47" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K29" s="42"/>
       <c r="L29" s="42"/>
     </row>
     <row r="30" ht="22.5" customHeight="1">
       <c r="A30" s="46" t="s">
-        <v>389</v>
+        <v>390</v>
       </c>
       <c r="B30" s="46" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="C30" s="45"/>
       <c r="D30" s="46" t="s">
@@ -22306,26 +22311,26 @@
       <c r="E30" s="45"/>
       <c r="F30" s="45"/>
       <c r="G30" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="H30" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="I30" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="J30" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K30" s="45"/>
       <c r="L30" s="45"/>
     </row>
     <row r="31" ht="22.5" customHeight="1">
       <c r="A31" s="47" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="B31" s="47" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="C31" s="42"/>
       <c r="D31" s="47" t="s">
@@ -22334,26 +22339,26 @@
       <c r="E31" s="42"/>
       <c r="F31" s="42"/>
       <c r="G31" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="H31" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="I31" s="47" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="J31" s="47" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K31" s="42"/>
       <c r="L31" s="42"/>
     </row>
     <row r="32" ht="22.5" customHeight="1">
       <c r="A32" s="46" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="B32" s="46" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="C32" s="45"/>
       <c r="D32" s="46" t="s">
@@ -22362,23 +22367,23 @@
       <c r="E32" s="45"/>
       <c r="F32" s="45"/>
       <c r="G32" s="46" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="H32" s="46" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="I32" s="49" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J32" s="49" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K32" s="50"/>
       <c r="L32" s="45"/>
     </row>
     <row r="33" ht="22.5" customHeight="1">
       <c r="A33" s="47" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B33" s="42"/>
       <c r="C33" s="42"/>
@@ -22391,14 +22396,14 @@
       <c r="H33" s="42"/>
       <c r="I33" s="42"/>
       <c r="J33" s="47" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="K33" s="42"/>
       <c r="L33" s="42"/>
     </row>
     <row r="34" ht="22.5" customHeight="1">
       <c r="A34" s="46" t="s">
-        <v>395</v>
+        <v>396</v>
       </c>
       <c r="B34" s="45"/>
       <c r="C34" s="45"/>
@@ -22411,17 +22416,17 @@
       <c r="H34" s="45"/>
       <c r="I34" s="45"/>
       <c r="J34" s="46" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K34" s="45"/>
       <c r="L34" s="45"/>
     </row>
     <row r="35" ht="22.5" customHeight="1">
       <c r="A35" s="47" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="B35" s="47" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="C35" s="42"/>
       <c r="D35" s="47" t="s">
@@ -22433,17 +22438,17 @@
       <c r="H35" s="42"/>
       <c r="I35" s="42"/>
       <c r="J35" s="47" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="K35" s="42"/>
       <c r="L35" s="42"/>
     </row>
     <row r="36" ht="22.5" customHeight="1">
       <c r="A36" s="46" t="s">
-        <v>398</v>
+        <v>399</v>
       </c>
       <c r="B36" s="46" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="C36" s="45"/>
       <c r="D36" s="46" t="s">
@@ -22456,16 +22461,16 @@
       <c r="I36" s="45"/>
       <c r="J36" s="45"/>
       <c r="K36" s="46" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="L36" s="45"/>
     </row>
     <row r="37" ht="22.5" customHeight="1">
       <c r="A37" s="47" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="B37" s="47" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="C37" s="42"/>
       <c r="D37" s="42"/>
@@ -22476,19 +22481,19 @@
       <c r="I37" s="42"/>
       <c r="J37" s="42"/>
       <c r="K37" s="47" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="L37" s="42"/>
     </row>
     <row r="38" ht="22.5" customHeight="1">
       <c r="A38" s="49" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B38" s="49" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="C38" s="52" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="D38" s="53" t="s">
         <v>8</v>
@@ -22498,11 +22503,11 @@
       <c r="G38" s="45"/>
       <c r="H38" s="45"/>
       <c r="I38" s="53" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="J38" s="50"/>
       <c r="K38" s="49" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="L38" s="45"/>
     </row>
@@ -22523,70 +22528,70 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="3" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="I1" s="3" t="s">
         <v>82</v>
       </c>
       <c r="J1" s="3" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="K1" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="L1" s="3" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>412</v>
+        <v>413</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="P1" s="3" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="Q1" s="3" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>419</v>
+        <v>420</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>423</v>
+        <v>424</v>
       </c>
       <c r="Y1" s="3" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="Z1" s="3" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
     </row>
     <row r="2">
@@ -22623,19 +22628,19 @@
         <v>-71.47352778</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="K2" s="3">
         <v>53.0</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M2" s="54" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Q2" s="3">
         <v>916626.0</v>
@@ -22644,10 +22649,10 @@
         <v>202175.0</v>
       </c>
       <c r="S2" s="3" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="T2" s="3" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="U2" s="3">
         <v>546632.0</v>
@@ -22656,10 +22661,10 @@
         <v>607006.0</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="X2" s="3" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="Y2" s="3">
         <v>-7956396.90869999</v>
@@ -22702,19 +22707,19 @@
         <v>-71.49854444</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="K3" s="3">
         <v>53.0</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M3" s="54" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Q3" s="3">
         <v>912582.0</v>
@@ -22723,10 +22728,10 @@
         <v>200119.0</v>
       </c>
       <c r="S3" s="3" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="T3" s="3" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="U3" s="3">
         <v>533365.0</v>
@@ -22735,10 +22740,10 @@
         <v>600259.0</v>
       </c>
       <c r="W3" s="3" t="s">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="X3" s="3" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="Y3" s="3">
         <v>-7959181.92299999</v>
@@ -22781,19 +22786,19 @@
         <v>-71.39156111</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="K4" s="3">
         <v>53.0</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M4" s="54" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Q4" s="3">
         <v>917369.0</v>
@@ -22802,10 +22807,10 @@
         <v>208912.0</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>441</v>
+        <v>442</v>
       </c>
       <c r="U4" s="3">
         <v>549070.0</v>
@@ -22814,10 +22819,10 @@
         <v>629107.0</v>
       </c>
       <c r="W4" s="3" t="s">
-        <v>442</v>
+        <v>443</v>
       </c>
       <c r="X4" s="3" t="s">
-        <v>443</v>
+        <v>444</v>
       </c>
       <c r="Y4" s="3">
         <v>-7947272.57209999</v>
@@ -22860,19 +22865,19 @@
         <v>-71.39794444</v>
       </c>
       <c r="I5" s="3" t="s">
-        <v>444</v>
+        <v>445</v>
       </c>
       <c r="J5" s="3" t="s">
-        <v>445</v>
+        <v>446</v>
       </c>
       <c r="K5" s="3">
         <v>53.0</v>
       </c>
       <c r="L5" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M5" s="54" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Q5" s="3">
         <v>919537.0</v>
@@ -22881,10 +22886,10 @@
         <v>208385.0</v>
       </c>
       <c r="S5" s="3" t="s">
-        <v>446</v>
+        <v>447</v>
       </c>
       <c r="T5" s="3" t="s">
-        <v>447</v>
+        <v>448</v>
       </c>
       <c r="U5" s="3">
         <v>556180.0</v>
@@ -22893,10 +22898,10 @@
         <v>627377.0</v>
       </c>
       <c r="W5" s="3" t="s">
-        <v>448</v>
+        <v>449</v>
       </c>
       <c r="X5" s="3" t="s">
-        <v>449</v>
+        <v>450</v>
       </c>
       <c r="Y5" s="3">
         <v>-7947983.11989999</v>
@@ -22939,19 +22944,19 @@
         <v>-71.38494444</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>450</v>
+        <v>451</v>
       </c>
       <c r="J6" s="3" t="s">
-        <v>451</v>
+        <v>452</v>
       </c>
       <c r="K6" s="3">
         <v>53.0</v>
       </c>
       <c r="L6" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M6" s="54" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Q6" s="3">
         <v>917108.0</v>
@@ -22960,10 +22965,10 @@
         <v>209456.0</v>
       </c>
       <c r="S6" s="3" t="s">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="T6" s="3" t="s">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="U6" s="3">
         <v>548214.0</v>
@@ -22972,10 +22977,10 @@
         <v>630892.0</v>
       </c>
       <c r="W6" s="3" t="s">
-        <v>454</v>
+        <v>455</v>
       </c>
       <c r="X6" s="3" t="s">
-        <v>455</v>
+        <v>456</v>
       </c>
       <c r="Y6" s="3">
         <v>-7946536.00149999</v>
@@ -23018,19 +23023,19 @@
         <v>-71.39951389</v>
       </c>
       <c r="I7" s="3" t="s">
-        <v>456</v>
+        <v>457</v>
       </c>
       <c r="J7" s="3" t="s">
-        <v>457</v>
+        <v>458</v>
       </c>
       <c r="K7" s="3">
         <v>53.0</v>
       </c>
       <c r="L7" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M7" s="54" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Q7" s="3">
         <v>920390.0</v>
@@ -23039,10 +23044,10 @@
         <v>208255.0</v>
       </c>
       <c r="S7" s="3" t="s">
-        <v>458</v>
+        <v>459</v>
       </c>
       <c r="T7" s="3" t="s">
-        <v>459</v>
+        <v>460</v>
       </c>
       <c r="U7" s="3">
         <v>558979.0</v>
@@ -23051,10 +23056,10 @@
         <v>626951.0</v>
       </c>
       <c r="W7" s="3" t="s">
-        <v>460</v>
+        <v>461</v>
       </c>
       <c r="X7" s="3" t="s">
-        <v>461</v>
+        <v>462</v>
       </c>
       <c r="Y7" s="3">
         <v>-7948157.69009999</v>
@@ -23097,19 +23102,19 @@
         <v>-71.43039167</v>
       </c>
       <c r="I8" s="3" t="s">
-        <v>462</v>
+        <v>463</v>
       </c>
       <c r="J8" s="3" t="s">
-        <v>463</v>
+        <v>464</v>
       </c>
       <c r="K8" s="3">
         <v>53.0</v>
       </c>
       <c r="L8" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M8" s="54" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Q8" s="3">
         <v>909604.0</v>
@@ -23118,10 +23123,10 @@
         <v>205727.0</v>
       </c>
       <c r="S8" s="3" t="s">
-        <v>464</v>
+        <v>465</v>
       </c>
       <c r="T8" s="3" t="s">
-        <v>465</v>
+        <v>466</v>
       </c>
       <c r="U8" s="3">
         <v>523592.0</v>
@@ -23130,10 +23135,10 @@
         <v>618657.0</v>
       </c>
       <c r="W8" s="3" t="s">
-        <v>466</v>
+        <v>467</v>
       </c>
       <c r="X8" s="3" t="s">
-        <v>467</v>
+        <v>468</v>
       </c>
       <c r="Y8" s="3">
         <v>-7951595.17399999</v>
@@ -23176,19 +23181,19 @@
         <v>-71.43501667</v>
       </c>
       <c r="I9" s="3" t="s">
-        <v>468</v>
+        <v>469</v>
       </c>
       <c r="J9" s="3" t="s">
-        <v>469</v>
+        <v>470</v>
       </c>
       <c r="K9" s="3">
         <v>53.0</v>
       </c>
       <c r="L9" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M9" s="54" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Q9" s="3">
         <v>919071.0</v>
@@ -23197,10 +23202,10 @@
         <v>205339.0</v>
       </c>
       <c r="S9" s="3" t="s">
-        <v>470</v>
+        <v>471</v>
       </c>
       <c r="T9" s="3" t="s">
-        <v>471</v>
+        <v>472</v>
       </c>
       <c r="U9" s="3">
         <v>554653.0</v>
@@ -23209,10 +23214,10 @@
         <v>617385.0</v>
       </c>
       <c r="W9" s="3" t="s">
-        <v>472</v>
+        <v>473</v>
       </c>
       <c r="X9" s="3" t="s">
-        <v>473</v>
+        <v>474</v>
       </c>
       <c r="Y9" s="3">
         <v>-7952109.8181</v>
@@ -23255,19 +23260,19 @@
         <v>-71.44393889</v>
       </c>
       <c r="I10" s="3" t="s">
-        <v>474</v>
+        <v>475</v>
       </c>
       <c r="J10" s="3" t="s">
-        <v>475</v>
+        <v>476</v>
       </c>
       <c r="K10" s="3">
         <v>53.0</v>
       </c>
       <c r="L10" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M10" s="54" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Q10" s="3">
         <v>917614.0</v>
@@ -23276,10 +23281,10 @@
         <v>204607.0</v>
       </c>
       <c r="S10" s="3" t="s">
-        <v>476</v>
+        <v>477</v>
       </c>
       <c r="T10" s="3" t="s">
-        <v>477</v>
+        <v>478</v>
       </c>
       <c r="U10" s="3">
         <v>549873.0</v>
@@ -23288,10 +23293,10 @@
         <v>614983.0</v>
       </c>
       <c r="W10" s="3" t="s">
-        <v>478</v>
+        <v>479</v>
       </c>
       <c r="X10" s="3" t="s">
-        <v>479</v>
+        <v>480</v>
       </c>
       <c r="Y10" s="3">
         <v>-7953103.0547</v>
@@ -23334,19 +23339,19 @@
         <v>-71.42853333</v>
       </c>
       <c r="I11" s="3" t="s">
-        <v>480</v>
+        <v>481</v>
       </c>
       <c r="J11" s="3" t="s">
-        <v>481</v>
+        <v>482</v>
       </c>
       <c r="K11" s="3">
         <v>53.0</v>
       </c>
       <c r="L11" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M11" s="54" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Q11" s="3">
         <v>919808.0</v>
@@ -23355,10 +23360,10 @@
         <v>205871.0</v>
       </c>
       <c r="S11" s="3" t="s">
-        <v>482</v>
+        <v>483</v>
       </c>
       <c r="T11" s="3" t="s">
-        <v>483</v>
+        <v>484</v>
       </c>
       <c r="U11" s="3">
         <v>557071.0</v>
@@ -23367,10 +23372,10 @@
         <v>619131.0</v>
       </c>
       <c r="W11" s="3" t="s">
-        <v>484</v>
+        <v>485</v>
       </c>
       <c r="X11" s="3" t="s">
-        <v>485</v>
+        <v>486</v>
       </c>
       <c r="Y11" s="3">
         <v>-7951388.09019999</v>
@@ -23413,19 +23418,19 @@
         <v>-71.46432778</v>
       </c>
       <c r="I12" s="3" t="s">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="J12" s="3" t="s">
-        <v>487</v>
+        <v>488</v>
       </c>
       <c r="K12" s="3">
         <v>53.0</v>
       </c>
       <c r="L12" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M12" s="54" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Q12" s="3">
         <v>911088.0</v>
@@ -23434,10 +23439,10 @@
         <v>202934.0</v>
       </c>
       <c r="S12" s="3" t="s">
-        <v>488</v>
+        <v>489</v>
       </c>
       <c r="T12" s="3" t="s">
-        <v>489</v>
+        <v>490</v>
       </c>
       <c r="U12" s="3">
         <v>528463.0</v>
@@ -23446,10 +23451,10 @@
         <v>609494.0</v>
       </c>
       <c r="W12" s="3" t="s">
-        <v>490</v>
+        <v>491</v>
       </c>
       <c r="X12" s="3" t="s">
-        <v>491</v>
+        <v>492</v>
       </c>
       <c r="Y12" s="3">
         <v>-7955372.7137</v>
@@ -23492,19 +23497,19 @@
         <v>-71.42379444</v>
       </c>
       <c r="I13" s="3" t="s">
-        <v>492</v>
+        <v>493</v>
       </c>
       <c r="J13" s="3" t="s">
-        <v>493</v>
+        <v>494</v>
       </c>
       <c r="K13" s="3">
         <v>53.0</v>
       </c>
       <c r="L13" s="3" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M13" s="54" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="Q13" s="3">
         <v>919518.0</v>
@@ -23513,10 +23518,10 @@
         <v>206261.0</v>
       </c>
       <c r="S13" s="3" t="s">
-        <v>494</v>
+        <v>495</v>
       </c>
       <c r="T13" s="3" t="s">
-        <v>495</v>
+        <v>496</v>
       </c>
       <c r="U13" s="3">
         <v>556120.0</v>
@@ -23525,10 +23530,10 @@
         <v>620409.0</v>
       </c>
       <c r="W13" s="3" t="s">
-        <v>496</v>
+        <v>497</v>
       </c>
       <c r="X13" s="3" t="s">
-        <v>497</v>
+        <v>498</v>
       </c>
       <c r="Y13" s="3">
         <v>-7950860.55109999</v>
@@ -23648,7 +23653,7 @@
         <v>Coordinate Source</v>
       </c>
       <c r="U1" s="6" t="s">
-        <v>498</v>
+        <v>499</v>
       </c>
       <c r="V1" s="38"/>
       <c r="W1" s="38"/>
@@ -25243,7 +25248,10 @@
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),45810.0)</f>
         <v>45810</v>
       </c>
-      <c r="Q28" s="5"/>
+      <c r="Q28" s="5" t="str">
+        <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"What we found is most likely the westerly of two monuments. The easterly monument would have been much closer to the actual boundary line. ")</f>
+        <v>What we found is most likely the westerly of two monuments. The easterly monument would have been much closer to the actual boundary line. </v>
+      </c>
       <c r="R28" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("""COMPUTED_VALUE"""),"The easterly and westerly sides of the Cash road")</f>
         <v>The easterly and westerly sides of the Cash road</v>
@@ -26619,13 +26627,13 @@
         <v>Longitude</v>
       </c>
       <c r="P1" s="6" t="s">
-        <v>499</v>
+        <v>500</v>
       </c>
       <c r="Q1" s="6" t="s">
-        <v>500</v>
+        <v>501</v>
       </c>
       <c r="R1" s="6" t="s">
-        <v>501</v>
+        <v>502</v>
       </c>
       <c r="S1" s="38"/>
       <c r="T1" s="38"/>
@@ -33037,24 +33045,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="61" t="s">
-        <v>502</v>
+        <v>503</v>
       </c>
       <c r="B1" s="61" t="s">
-        <v>503</v>
+        <v>504</v>
       </c>
       <c r="C1" s="61" t="s">
-        <v>504</v>
+        <v>505</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>505</v>
+        <v>506</v>
       </c>
       <c r="E1" s="8" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="8" t="s">
-        <v>506</v>
+        <v>507</v>
       </c>
       <c r="B2" s="5" t="str">
         <f t="array" ref="B2">index($G$14:BO$14,0,MATCH(MIN(ABS(G2:R2)), ABS(G2:R2),0))</f>
@@ -33123,7 +33131,7 @@
     </row>
     <row r="3">
       <c r="A3" s="8" t="s">
-        <v>507</v>
+        <v>508</v>
       </c>
       <c r="B3" s="5" t="str">
         <f t="array" ref="B3">index($G$14:BO$14,0,MATCH(MIN(ABS(G3:R3)), ABS(G3:R3),0))</f>
@@ -33192,7 +33200,7 @@
     </row>
     <row r="4">
       <c r="A4" s="8" t="s">
-        <v>508</v>
+        <v>509</v>
       </c>
       <c r="B4" s="5" t="str">
         <f t="array" ref="B4">index($G$14:BO$14,0,MATCH(MIN(ABS(G4:R4)), ABS(G4:R4),0))</f>
@@ -33261,7 +33269,7 @@
     </row>
     <row r="5">
       <c r="A5" s="8" t="s">
-        <v>509</v>
+        <v>510</v>
       </c>
       <c r="B5" s="5" t="str">
         <f t="array" ref="B5">index($G$14:BO$14,0,MATCH(MIN(ABS(G5:R5)), ABS(G5:R5),0))</f>
@@ -33330,7 +33338,7 @@
     </row>
     <row r="6">
       <c r="A6" s="8" t="s">
-        <v>510</v>
+        <v>511</v>
       </c>
       <c r="B6" s="5" t="str">
         <f t="array" ref="B6">index($G$14:BO$14,0,MATCH(MIN(ABS(G6:R6)), ABS(G6:R6),0))</f>
@@ -33399,7 +33407,7 @@
     </row>
     <row r="7">
       <c r="A7" s="8" t="s">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="B7" s="5" t="str">
         <f t="array" ref="B7">index($G$14:BO$14,0,MATCH(MIN(ABS(G7:R7)), ABS(G7:R7),0))</f>
@@ -33468,7 +33476,7 @@
     </row>
     <row r="8">
       <c r="A8" s="8" t="s">
-        <v>512</v>
+        <v>513</v>
       </c>
       <c r="B8" s="5" t="str">
         <f t="array" ref="B8">index($G$14:BO$14,0,MATCH(MIN(ABS(G8:R8)), ABS(G8:R8),0))</f>
@@ -33537,7 +33545,7 @@
     </row>
     <row r="9">
       <c r="A9" s="8" t="s">
-        <v>513</v>
+        <v>514</v>
       </c>
       <c r="B9" s="5" t="str">
         <f t="array" ref="B9">index($G$14:BO$14,0,MATCH(MIN(ABS(G9:R9)), ABS(G9:R9),0))</f>
@@ -33606,7 +33614,7 @@
     </row>
     <row r="10">
       <c r="A10" s="8" t="s">
-        <v>514</v>
+        <v>515</v>
       </c>
       <c r="B10" s="5" t="str">
         <f t="array" ref="B10">index($G$14:BO$14,0,MATCH(MIN(ABS(G10:R10)), ABS(G10:R10),0))</f>
@@ -33675,7 +33683,7 @@
     </row>
     <row r="11">
       <c r="A11" s="8" t="s">
-        <v>515</v>
+        <v>516</v>
       </c>
       <c r="B11" s="5" t="str">
         <f t="array" ref="B11">index($G$14:BO$14,0,MATCH(MIN(ABS(G11:R11)), ABS(G11:R11),0))</f>
@@ -33744,7 +33752,7 @@
     </row>
     <row r="12">
       <c r="A12" s="8" t="s">
-        <v>516</v>
+        <v>517</v>
       </c>
       <c r="B12" s="5" t="str">
         <f t="array" ref="B12">index($G$14:BO$14,0,MATCH(MIN(ABS(G12:R12)), ABS(G12:R12),0))</f>
@@ -33813,7 +33821,7 @@
     </row>
     <row r="13">
       <c r="A13" s="8" t="s">
-        <v>517</v>
+        <v>518</v>
       </c>
       <c r="B13" s="5" t="str">
         <f t="array" ref="B13">index($G$14:BO$14,0,MATCH(MIN(ABS(G13:R13)), ABS(G13:R13),0))</f>
@@ -33886,7 +33894,7 @@
       <c r="D14" s="8"/>
       <c r="E14" s="8"/>
       <c r="F14" s="3" t="s">
-        <v>518</v>
+        <v>519</v>
       </c>
       <c r="G14" s="5" t="str">
         <f>IFERROR(__xludf.DUMMYFUNCTION("transpose(filter(Monuments!A$2:A918,Monuments!B2:B918=""Corner""))"),"Acton/Boxborough/Littleton")</f>
@@ -33939,7 +33947,7 @@
       <c r="D15" s="8"/>
       <c r="E15" s="8"/>
       <c r="F15" s="3" t="s">
-        <v>519</v>
+        <v>520</v>
       </c>
       <c r="G15" s="3">
         <f>IFERROR(__xludf.DUMMYFUNCTION("transpose(filter(Monuments!X$2:X918,Monuments!B2:B918=""Corner""))"),-71.473529496)</f>
@@ -33992,7 +34000,7 @@
       <c r="D16" s="8"/>
       <c r="E16" s="8"/>
       <c r="F16" s="3" t="s">
-        <v>520</v>
+        <v>521</v>
       </c>
       <c r="G16" s="63">
         <f>IFERROR(__xludf.DUMMYFUNCTION("transpose(filter(Monuments!T$2:T918,Monuments!B2:B918=""Corner""))"),42.5001860150001)</f>
@@ -34041,7 +34049,7 @@
     </row>
     <row r="17">
       <c r="F17" s="3" t="s">
-        <v>521</v>
+        <v>522</v>
       </c>
       <c r="G17" s="5" t="str">
         <f t="shared" ref="G17:R17" si="15">vlookup(G$14,$B:$E,4,False)</f>
@@ -34094,7 +34102,7 @@
     </row>
     <row r="18">
       <c r="F18" s="3" t="s">
-        <v>522</v>
+        <v>523</v>
       </c>
       <c r="G18" s="5" t="str">
         <f t="shared" ref="G18:R18" si="16">vlookup(G$14,$B:$E,3,False)</f>
@@ -34147,7 +34155,7 @@
     </row>
     <row r="19">
       <c r="F19" s="3" t="s">
-        <v>523</v>
+        <v>524</v>
       </c>
       <c r="G19" s="64">
         <f t="shared" ref="G19:R19" si="17">G17-G15</f>
@@ -34200,7 +34208,7 @@
     </row>
     <row r="20">
       <c r="F20" s="3" t="s">
-        <v>524</v>
+        <v>525</v>
       </c>
       <c r="G20" s="64">
         <f t="shared" ref="G20:R20" si="18">G18-G16</f>
@@ -34281,7 +34289,7 @@
     </row>
     <row r="2">
       <c r="A2" s="3" t="s">
-        <v>525</v>
+        <v>526</v>
       </c>
       <c r="B2" s="22">
         <v>42.5001860150001</v>
@@ -34292,7 +34300,7 @@
     </row>
     <row r="3">
       <c r="A3" s="3" t="s">
-        <v>526</v>
+        <v>527</v>
       </c>
       <c r="B3" s="22">
         <v>42.4637837510001</v>
@@ -34303,7 +34311,7 @@
     </row>
     <row r="4">
       <c r="A4" s="3" t="s">
-        <v>527</v>
+        <v>528</v>
       </c>
       <c r="B4" s="22">
         <v>42.5068287080001</v>
@@ -34314,7 +34322,7 @@
     </row>
     <row r="5">
       <c r="A5" s="3" t="s">
-        <v>528</v>
+        <v>529</v>
       </c>
       <c r="B5" s="22">
         <v>42.526344807</v>
@@ -34325,7 +34333,7 @@
     </row>
     <row r="6">
       <c r="A6" s="3" t="s">
-        <v>529</v>
+        <v>530</v>
       </c>
       <c r="B6" s="22">
         <v>42.504473137</v>
@@ -34336,7 +34344,7 @@
     </row>
     <row r="7">
       <c r="A7" s="3" t="s">
-        <v>530</v>
+        <v>531</v>
       </c>
       <c r="B7" s="22">
         <v>42.534025086</v>
@@ -34347,7 +34355,7 @@
     </row>
     <row r="8">
       <c r="A8" s="3" t="s">
-        <v>531</v>
+        <v>532</v>
       </c>
       <c r="B8" s="22">
         <v>42.436947994</v>
@@ -34358,7 +34366,7 @@
     </row>
     <row r="9">
       <c r="A9" s="3" t="s">
-        <v>532</v>
+        <v>533</v>
       </c>
       <c r="B9" s="22">
         <v>42.5221791480001</v>
@@ -34369,7 +34377,7 @@
     </row>
     <row r="10">
       <c r="A10" s="3" t="s">
-        <v>533</v>
+        <v>534</v>
       </c>
       <c r="B10" s="22">
         <v>42.509068563</v>
@@ -34380,7 +34388,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="s">
-        <v>534</v>
+        <v>535</v>
       </c>
       <c r="B11" s="22">
         <v>42.528812154</v>
@@ -34391,7 +34399,7 @@
     </row>
     <row r="12">
       <c r="A12" s="3" t="s">
-        <v>535</v>
+        <v>536</v>
       </c>
       <c r="B12" s="22">
         <v>42.4503286410001</v>
@@ -34402,7 +34410,7 @@
     </row>
     <row r="13">
       <c r="A13" s="3" t="s">
-        <v>536</v>
+        <v>537</v>
       </c>
       <c r="B13" s="22">
         <v>42.5261982760001</v>

</xml_diff>